<commit_message>
NCD_Brand_Tagging: Cup (14oz) แท็กเป็น shared
แพรยืนยัน — ใช้ทั้ง YC และ Staple (ไม่ใช่ YC อย่างเดียวเหมือนที่ตั้งไว้ก่อน)
Par NCD ยังเว้นว่างไว้เหมือนเดิม รอแพรกรอกจำนวนจริง
</commit_message>
<xml_diff>
--- a/NCD_Brand_Tagging.xlsx
+++ b/NCD_Brand_Tagging.xlsx
@@ -2,9 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="660" windowWidth="29400" windowHeight="17220" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Instructions" sheetId="1" state="visible" r:id="rId1"/>
@@ -12,7 +11,7 @@
     <sheet name="New Staple Items" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="0" fullCalcOnLoad="1" iterateDelta="0.0001"/>
 </workbook>
 </file>
 
@@ -29,40 +28,47 @@
     </font>
     <font>
       <name val="Arial"/>
+      <family val="2"/>
       <b val="1"/>
-      <color rgb="00542916"/>
+      <color rgb="FF542916"/>
       <sz val="14"/>
     </font>
     <font>
       <name val="Arial"/>
-      <color rgb="002B241C"/>
+      <family val="2"/>
+      <color rgb="FF2B241C"/>
       <sz val="10"/>
     </font>
     <font>
       <name val="Arial"/>
-      <color rgb="002B241C"/>
+      <family val="2"/>
+      <color rgb="FF2B241C"/>
       <sz val="11"/>
     </font>
     <font>
       <name val="Arial"/>
+      <family val="2"/>
       <b val="1"/>
-      <color rgb="00542916"/>
+      <color rgb="FF542916"/>
       <sz val="11"/>
     </font>
     <font>
       <name val="Arial"/>
+      <family val="2"/>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
+      <color rgb="FFFFFFFF"/>
       <sz val="11"/>
     </font>
     <font>
       <name val="Arial"/>
+      <family val="2"/>
       <sz val="10"/>
     </font>
     <font>
       <name val="Arial"/>
+      <family val="2"/>
       <i val="1"/>
-      <color rgb="00808080"/>
+      <color rgb="FF808080"/>
       <sz val="10"/>
     </font>
   </fonts>
@@ -75,14 +81,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F2565C"/>
-        <bgColor rgb="00F2565C"/>
+        <fgColor rgb="FFF2565C"/>
+        <bgColor rgb="FFF2565C"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFF9C4"/>
-        <bgColor rgb="00FFF9C4"/>
+        <fgColor rgb="FFFFF9C4"/>
+        <bgColor rgb="FFFFF9C4"/>
       </patternFill>
     </fill>
   </fills>
@@ -96,17 +102,18 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="00D9D9D9"/>
+        <color rgb="FFD9D9D9"/>
       </left>
       <right style="thin">
-        <color rgb="00D9D9D9"/>
+        <color rgb="FFD9D9D9"/>
       </right>
       <top style="thin">
-        <color rgb="00D9D9D9"/>
+        <color rgb="FFD9D9D9"/>
       </top>
       <bottom style="thin">
-        <color rgb="00D9D9D9"/>
+        <color rgb="FFD9D9D9"/>
       </bottom>
+      <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
@@ -149,7 +156,7 @@
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -533,7 +540,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:A26"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
   </cols>
@@ -546,7 +553,7 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr"/>
+      <c r="A2" s="2" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
@@ -570,7 +577,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="inlineStr"/>
+      <c r="A6" s="2" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
@@ -657,7 +664,7 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="2" t="inlineStr"/>
+      <c r="A19" s="2" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
@@ -695,7 +702,7 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="2" t="inlineStr"/>
+      <c r="A25" s="2" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="4" t="inlineStr">
@@ -716,7 +723,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:J119"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
@@ -725,9 +732,7 @@
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="22" customWidth="1" min="6" max="6"/>
     <col width="30" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
-    <col width="12" customWidth="1" min="9" max="9"/>
-    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="8" max="10"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -806,7 +811,9 @@
           <t>1kg/Box</t>
         </is>
       </c>
-      <c r="F2" s="8" t="n"/>
+      <c r="F2" s="8" t="n">
+        <v>3</v>
+      </c>
       <c r="G2" s="8" t="inlineStr">
         <is>
           <t>yc</t>
@@ -846,7 +853,9 @@
           <t>1kg/Box</t>
         </is>
       </c>
-      <c r="F3" s="8" t="n"/>
+      <c r="F3" s="8" t="n">
+        <v>1</v>
+      </c>
       <c r="G3" s="8" t="inlineStr">
         <is>
           <t>yc</t>
@@ -1126,7 +1135,9 @@
           <t>1kg/Box</t>
         </is>
       </c>
-      <c r="F10" s="8" t="n"/>
+      <c r="F10" s="8" t="n">
+        <v>3</v>
+      </c>
       <c r="G10" s="8" t="inlineStr">
         <is>
           <t>yc</t>
@@ -1166,7 +1177,9 @@
           <t>500g/Box</t>
         </is>
       </c>
-      <c r="F11" s="8" t="n"/>
+      <c r="F11" s="8" t="n">
+        <v>5</v>
+      </c>
       <c r="G11" s="8" t="inlineStr">
         <is>
           <t>yc</t>
@@ -1206,7 +1219,9 @@
           <t>500g/Box</t>
         </is>
       </c>
-      <c r="F12" s="8" t="n"/>
+      <c r="F12" s="8" t="n">
+        <v>5</v>
+      </c>
       <c r="G12" s="8" t="inlineStr">
         <is>
           <t>yc</t>
@@ -1432,7 +1447,9 @@
           <t>ถ้วย</t>
         </is>
       </c>
-      <c r="F18" s="8" t="n"/>
+      <c r="F18" s="8" t="n">
+        <v>40</v>
+      </c>
       <c r="G18" s="8" t="inlineStr">
         <is>
           <t>yc</t>
@@ -1504,7 +1521,9 @@
           <t>ขวด</t>
         </is>
       </c>
-      <c r="F20" s="8" t="n"/>
+      <c r="F20" s="8" t="n">
+        <v>12</v>
+      </c>
       <c r="G20" s="8" t="inlineStr">
         <is>
           <t>yc</t>
@@ -1542,7 +1561,9 @@
           <t>ถุง</t>
         </is>
       </c>
-      <c r="F21" s="8" t="n"/>
+      <c r="F21" s="8" t="n">
+        <v>5</v>
+      </c>
       <c r="G21" s="8" t="inlineStr">
         <is>
           <t>yc</t>
@@ -1582,7 +1603,9 @@
           <t>ถุง</t>
         </is>
       </c>
-      <c r="F22" s="8" t="n"/>
+      <c r="F22" s="8" t="n">
+        <v>5</v>
+      </c>
       <c r="G22" s="8" t="inlineStr">
         <is>
           <t>yc</t>
@@ -1622,7 +1645,9 @@
           <t>ถุง</t>
         </is>
       </c>
-      <c r="F23" s="8" t="n"/>
+      <c r="F23" s="8" t="n">
+        <v>5</v>
+      </c>
       <c r="G23" s="8" t="inlineStr">
         <is>
           <t>yc</t>
@@ -1662,7 +1687,9 @@
           <t>ถุง</t>
         </is>
       </c>
-      <c r="F24" s="8" t="n"/>
+      <c r="F24" s="8" t="n">
+        <v>5</v>
+      </c>
       <c r="G24" s="8" t="inlineStr">
         <is>
           <t>yc</t>
@@ -1702,7 +1729,9 @@
           <t>ถุง</t>
         </is>
       </c>
-      <c r="F25" s="8" t="n"/>
+      <c r="F25" s="8" t="n">
+        <v>5</v>
+      </c>
       <c r="G25" s="8" t="inlineStr">
         <is>
           <t>yc</t>
@@ -1742,7 +1771,9 @@
           <t>ถุง</t>
         </is>
       </c>
-      <c r="F26" s="8" t="n"/>
+      <c r="F26" s="8" t="n">
+        <v>5</v>
+      </c>
       <c r="G26" s="8" t="inlineStr">
         <is>
           <t>yc</t>
@@ -1782,7 +1813,9 @@
           <t>กระปุก</t>
         </is>
       </c>
-      <c r="F27" s="8" t="n"/>
+      <c r="F27" s="8" t="n">
+        <v>5</v>
+      </c>
       <c r="G27" s="8" t="inlineStr">
         <is>
           <t>yc</t>
@@ -1820,7 +1853,9 @@
           <t>กระปุก</t>
         </is>
       </c>
-      <c r="F28" s="8" t="n"/>
+      <c r="F28" s="8" t="n">
+        <v>5</v>
+      </c>
       <c r="G28" s="8" t="inlineStr">
         <is>
           <t>yc</t>
@@ -1858,7 +1893,9 @@
           <t>กระปุก</t>
         </is>
       </c>
-      <c r="F29" s="8" t="n"/>
+      <c r="F29" s="8" t="n">
+        <v>5</v>
+      </c>
       <c r="G29" s="8" t="inlineStr">
         <is>
           <t>yc</t>
@@ -1896,7 +1933,9 @@
           <t>750g/pack</t>
         </is>
       </c>
-      <c r="F30" s="8" t="n"/>
+      <c r="F30" s="8" t="n">
+        <v>2</v>
+      </c>
       <c r="G30" s="8" t="inlineStr">
         <is>
           <t>yc</t>
@@ -1936,7 +1975,9 @@
           <t>454g/pack</t>
         </is>
       </c>
-      <c r="F31" s="8" t="n"/>
+      <c r="F31" s="8" t="n">
+        <v>2</v>
+      </c>
       <c r="G31" s="8" t="inlineStr">
         <is>
           <t>yc</t>
@@ -1976,7 +2017,9 @@
           <t>300g/pack</t>
         </is>
       </c>
-      <c r="F32" s="8" t="n"/>
+      <c r="F32" s="8" t="n">
+        <v>1</v>
+      </c>
       <c r="G32" s="8" t="inlineStr">
         <is>
           <t>yc</t>
@@ -2016,7 +2059,9 @@
           <t>1,000g/box</t>
         </is>
       </c>
-      <c r="F33" s="8" t="n"/>
+      <c r="F33" s="8" t="n">
+        <v>1</v>
+      </c>
       <c r="G33" s="8" t="inlineStr">
         <is>
           <t>yc</t>
@@ -2056,7 +2101,9 @@
           <t>2,000g/box</t>
         </is>
       </c>
-      <c r="F34" s="8" t="n"/>
+      <c r="F34" s="8" t="n">
+        <v>1</v>
+      </c>
       <c r="G34" s="8" t="inlineStr">
         <is>
           <t>yc</t>
@@ -2096,7 +2143,9 @@
           <t>400g/pack</t>
         </is>
       </c>
-      <c r="F35" s="8" t="n"/>
+      <c r="F35" s="8" t="n">
+        <v>1</v>
+      </c>
       <c r="G35" s="8" t="inlineStr">
         <is>
           <t>yc</t>
@@ -2134,7 +2183,9 @@
           <t>400g/pack</t>
         </is>
       </c>
-      <c r="F36" s="8" t="n"/>
+      <c r="F36" s="8" t="n">
+        <v>1</v>
+      </c>
       <c r="G36" s="8" t="inlineStr">
         <is>
           <t>yc</t>
@@ -2172,7 +2223,9 @@
           <t>400g/pack</t>
         </is>
       </c>
-      <c r="F37" s="8" t="n"/>
+      <c r="F37" s="8" t="n">
+        <v>1</v>
+      </c>
       <c r="G37" s="8" t="inlineStr">
         <is>
           <t>yc</t>
@@ -2248,7 +2301,9 @@
           <t>400g/pack</t>
         </is>
       </c>
-      <c r="F39" s="8" t="n"/>
+      <c r="F39" s="8" t="n">
+        <v>1</v>
+      </c>
       <c r="G39" s="8" t="inlineStr">
         <is>
           <t>yc</t>
@@ -2288,7 +2343,9 @@
           <t>400g/pack</t>
         </is>
       </c>
-      <c r="F40" s="8" t="n"/>
+      <c r="F40" s="8" t="n">
+        <v>1</v>
+      </c>
       <c r="G40" s="8" t="inlineStr">
         <is>
           <t>yc</t>
@@ -2328,7 +2385,9 @@
           <t>400g/pack</t>
         </is>
       </c>
-      <c r="F41" s="8" t="n"/>
+      <c r="F41" s="8" t="n">
+        <v>1</v>
+      </c>
       <c r="G41" s="8" t="inlineStr">
         <is>
           <t>yc</t>
@@ -2368,7 +2427,9 @@
           <t>1,000g/pack</t>
         </is>
       </c>
-      <c r="F42" s="8" t="n"/>
+      <c r="F42" s="8" t="n">
+        <v>1</v>
+      </c>
       <c r="G42" s="8" t="inlineStr">
         <is>
           <t>yc</t>
@@ -2406,7 +2467,9 @@
           <t>1,000g/pack</t>
         </is>
       </c>
-      <c r="F43" s="8" t="n"/>
+      <c r="F43" s="8" t="n">
+        <v>1</v>
+      </c>
       <c r="G43" s="8" t="inlineStr">
         <is>
           <t>yc</t>
@@ -2444,7 +2507,9 @@
           <t>250g/box</t>
         </is>
       </c>
-      <c r="F44" s="8" t="n"/>
+      <c r="F44" s="8" t="n">
+        <v>3</v>
+      </c>
       <c r="G44" s="8" t="inlineStr">
         <is>
           <t>yc</t>
@@ -2552,7 +2617,9 @@
           <t>300g/box</t>
         </is>
       </c>
-      <c r="F47" s="8" t="n"/>
+      <c r="F47" s="8" t="n">
+        <v>2</v>
+      </c>
       <c r="G47" s="8" t="inlineStr">
         <is>
           <t>yc</t>
@@ -2626,7 +2693,9 @@
           <t>500g/pack</t>
         </is>
       </c>
-      <c r="F49" s="8" t="n"/>
+      <c r="F49" s="8" t="n">
+        <v>1</v>
+      </c>
       <c r="G49" s="8" t="inlineStr">
         <is>
           <t>yc</t>
@@ -2666,7 +2735,9 @@
           <t>ลูก</t>
         </is>
       </c>
-      <c r="F50" s="8" t="n"/>
+      <c r="F50" s="8" t="n">
+        <v>6</v>
+      </c>
       <c r="G50" s="8" t="inlineStr">
         <is>
           <t>yc</t>
@@ -2706,7 +2777,9 @@
           <t>1,000g/bottle</t>
         </is>
       </c>
-      <c r="F51" s="8" t="n"/>
+      <c r="F51" s="8" t="n">
+        <v>2</v>
+      </c>
       <c r="G51" s="8" t="inlineStr">
         <is>
           <t>yc</t>
@@ -2746,7 +2819,9 @@
           <t>1,000g/bottle</t>
         </is>
       </c>
-      <c r="F52" s="8" t="n"/>
+      <c r="F52" s="8" t="n">
+        <v>2</v>
+      </c>
       <c r="G52" s="8" t="inlineStr">
         <is>
           <t>yc</t>
@@ -2786,7 +2861,9 @@
           <t>1,000g/pack</t>
         </is>
       </c>
-      <c r="F53" s="8" t="n"/>
+      <c r="F53" s="8" t="n">
+        <v>2</v>
+      </c>
       <c r="G53" s="8" t="inlineStr">
         <is>
           <t>yc</t>
@@ -2906,7 +2983,9 @@
           <t>50/pack</t>
         </is>
       </c>
-      <c r="F56" s="8" t="n"/>
+      <c r="F56" s="8" t="n">
+        <v>2</v>
+      </c>
       <c r="G56" s="8" t="inlineStr">
         <is>
           <t>yc</t>
@@ -2949,7 +3028,7 @@
       <c r="F57" s="8" t="n"/>
       <c r="G57" s="8" t="inlineStr">
         <is>
-          <t>yc</t>
+          <t>shared</t>
         </is>
       </c>
       <c r="H57" s="6" t="n">
@@ -2986,10 +3065,12 @@
           <t>50/pack</t>
         </is>
       </c>
-      <c r="F58" s="8" t="n"/>
+      <c r="F58" s="8" t="n">
+        <v>2</v>
+      </c>
       <c r="G58" s="8" t="inlineStr">
         <is>
-          <t>yc</t>
+          <t>shared</t>
         </is>
       </c>
       <c r="H58" s="6" t="n">
@@ -3026,10 +3107,12 @@
           <t>50/pack</t>
         </is>
       </c>
-      <c r="F59" s="8" t="n"/>
+      <c r="F59" s="8" t="n">
+        <v>2</v>
+      </c>
       <c r="G59" s="8" t="inlineStr">
         <is>
-          <t>yc</t>
+          <t>shared</t>
         </is>
       </c>
       <c r="H59" s="6" t="n">
@@ -3066,10 +3149,12 @@
           <t>50/pack</t>
         </is>
       </c>
-      <c r="F60" s="8" t="n"/>
+      <c r="F60" s="8" t="n">
+        <v>2</v>
+      </c>
       <c r="G60" s="8" t="inlineStr">
         <is>
-          <t>yc</t>
+          <t>shared</t>
         </is>
       </c>
       <c r="H60" s="6" t="n">
@@ -3106,7 +3191,9 @@
           <t>50/pack</t>
         </is>
       </c>
-      <c r="F61" s="8" t="n"/>
+      <c r="F61" s="8" t="n">
+        <v>2</v>
+      </c>
       <c r="G61" s="8" t="inlineStr">
         <is>
           <t>yc</t>
@@ -3146,7 +3233,9 @@
           <t>50/pack</t>
         </is>
       </c>
-      <c r="F62" s="8" t="n"/>
+      <c r="F62" s="8" t="n">
+        <v>2</v>
+      </c>
       <c r="G62" s="8" t="inlineStr">
         <is>
           <t>yc</t>
@@ -3226,10 +3315,12 @@
           <t>50/pack</t>
         </is>
       </c>
-      <c r="F64" s="8" t="n"/>
+      <c r="F64" s="8" t="n">
+        <v>2</v>
+      </c>
       <c r="G64" s="8" t="inlineStr">
         <is>
-          <t>yc</t>
+          <t>shared</t>
         </is>
       </c>
       <c r="H64" s="6" t="n">
@@ -3266,10 +3357,12 @@
           <t>100/pack</t>
         </is>
       </c>
-      <c r="F65" s="8" t="n"/>
+      <c r="F65" s="8" t="n">
+        <v>2</v>
+      </c>
       <c r="G65" s="8" t="inlineStr">
         <is>
-          <t>yc</t>
+          <t>shared</t>
         </is>
       </c>
       <c r="H65" s="6" t="n">
@@ -3306,10 +3399,12 @@
           <t>100/pack</t>
         </is>
       </c>
-      <c r="F66" s="8" t="n"/>
+      <c r="F66" s="8" t="n">
+        <v>5</v>
+      </c>
       <c r="G66" s="8" t="inlineStr">
         <is>
-          <t>yc</t>
+          <t>shared</t>
         </is>
       </c>
       <c r="H66" s="6" t="n">
@@ -3346,10 +3441,12 @@
           <t>100/pack</t>
         </is>
       </c>
-      <c r="F67" s="8" t="n"/>
+      <c r="F67" s="8" t="n">
+        <v>1</v>
+      </c>
       <c r="G67" s="8" t="inlineStr">
         <is>
-          <t>yc</t>
+          <t>shared</t>
         </is>
       </c>
       <c r="H67" s="6" t="n">
@@ -3429,7 +3526,7 @@
       <c r="F69" s="8" t="n"/>
       <c r="G69" s="8" t="inlineStr">
         <is>
-          <t>yc</t>
+          <t>shared</t>
         </is>
       </c>
       <c r="H69" s="6" t="n">
@@ -3469,7 +3566,7 @@
       <c r="F70" s="8" t="n"/>
       <c r="G70" s="8" t="inlineStr">
         <is>
-          <t>yc</t>
+          <t>staple</t>
         </is>
       </c>
       <c r="H70" s="6" t="n">
@@ -5272,7 +5369,9 @@
           <t>กระปุก</t>
         </is>
       </c>
-      <c r="F117" s="8" t="n"/>
+      <c r="F117" s="8" t="n">
+        <v>5</v>
+      </c>
       <c r="G117" s="8" t="inlineStr">
         <is>
           <t>yc</t>
@@ -5380,7 +5479,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:F42"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
     <col width="34" customWidth="1" min="2" max="2"/>
@@ -5422,7 +5521,7 @@
         </is>
       </c>
     </row>
-    <row r="2">
+    <row r="2" ht="28" customHeight="1">
       <c r="A2" s="9" t="n">
         <v>1</v>
       </c>

</xml_diff>

<commit_message>
NCD_Brand_Tagging: เปลี่ยนชื่อถุง + ลบ Large เพิ่ม S/M Brown Paper Bag
แพรแก้ 2026-08-05 — ตัดคำว่า "NCD" กับ "(new design)" ออกจากชื่อถุง
เดี่ยว/คู่ (ชื่อยาวเกินจำเป็น) ลบ "Large Paper Bag" ออก แทนที่ด้วย
S Brown Paper Bag และ M Brown Paper Bag แยก 2 ขนาด — ทั้งคู่ตั้ง brand
shared ตามบริบทชุดเดียวกับถุงเดี่ยว/คู่ รอแพรกรอก Par NCD
</commit_message>
<xml_diff>
--- a/NCD_Brand_Tagging.xlsx
+++ b/NCD_Brand_Tagging.xlsx
@@ -5725,7 +5725,7 @@
       </c>
       <c r="B4" s="8" t="inlineStr">
         <is>
-          <t>NCD Single Cup Paper Bag (new design)</t>
+          <t>Single Cup Paper Bag</t>
         </is>
       </c>
       <c r="C4" s="8" t="inlineStr">
@@ -5756,7 +5756,7 @@
       </c>
       <c r="B5" s="8" t="inlineStr">
         <is>
-          <t>NCD Double Cup Paper Bag (new design)</t>
+          <t>Double Cup Paper Bag</t>
         </is>
       </c>
       <c r="C5" s="8" t="inlineStr">
@@ -5787,7 +5787,7 @@
       </c>
       <c r="B6" s="8" t="inlineStr">
         <is>
-          <t>NCD Large Paper Bag (new design)</t>
+          <t>S Brown Paper Bag</t>
         </is>
       </c>
       <c r="C6" s="8" t="inlineStr">
@@ -5808,7 +5808,7 @@
       <c r="F6" s="9" t="n"/>
       <c r="G6" s="8" t="inlineStr">
         <is>
-          <t>New bag design used ONLY at NCD, shared by both YC and Staple. NOT the same item as YC's existing ถุงกระดาษใหญ่ (it-073) used at NVP/SND/KCN — that one stays a separate, unrelated item. Fill in Par NCD.</t>
+          <t>New NCD-only bag, shared by both YC and Staple. Fill in Par NCD.</t>
         </is>
       </c>
     </row>
@@ -5816,12 +5816,32 @@
       <c r="A7" s="9" t="n">
         <v>6</v>
       </c>
-      <c r="B7" s="8" t="n"/>
-      <c r="C7" s="8" t="n"/>
-      <c r="D7" s="8" t="n"/>
-      <c r="E7" s="8" t="n"/>
+      <c r="B7" s="8" t="inlineStr">
+        <is>
+          <t>M Brown Paper Bag</t>
+        </is>
+      </c>
+      <c r="C7" s="8" t="inlineStr">
+        <is>
+          <t>Bags</t>
+        </is>
+      </c>
+      <c r="D7" s="8" t="inlineStr">
+        <is>
+          <t>ใบ</t>
+        </is>
+      </c>
+      <c r="E7" s="8" t="inlineStr">
+        <is>
+          <t>shared</t>
+        </is>
+      </c>
       <c r="F7" s="9" t="n"/>
-      <c r="G7" s="8" t="n"/>
+      <c r="G7" s="8" t="inlineStr">
+        <is>
+          <t>New NCD-only bag, shared by both YC and Staple. Fill in Par NCD.</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="9" t="n">

</xml_diff>

<commit_message>
NCD_Brand_Tagging: เพิ่ม 10 สินค้าใหม่ในหมวด To-Go (Cheese/Sandwich & Salad/Beverage)
แก้เฉพาะจุด (เติมแถวว่างที่มีอยู่แล้วในชีต ไม่ regenerate) ตามรายชื่อที่แพรส่งมา:
- To-Go Cheese: Feta Cheese, Ricotta (กระปุก)
- To-Go Sandwich & Salad: Ham Cheese/Egg Salad/Tuna Sandwich (ชิ้น)
- To-Go Beverage: Sour Hour Ginger Lemon/Peach Lychee, Coca Cola, Sprite (กระป๋อง),
  San Pellegrino (ขวด — เจ้าเดียวที่เป็นขวดไม่ใช่กระป๋อง)
ทั้งหมด brand=shared (แพรยืนยัน) · "Drinking Water" ไม่เพิ่มซ้ำ เพราะเป็นตัวเดียวกับ
Water น้ำดื่ม (it-019) ที่แท็ก To-Go Beverage ไว้แล้วในชีต Existing Items

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/NCD_Brand_Tagging.xlsx
+++ b/NCD_Brand_Tagging.xlsx
@@ -2,9 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="660" windowWidth="29400" windowHeight="17220" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Instructions" sheetId="1" state="visible" r:id="rId1"/>
@@ -12,7 +11,7 @@
     <sheet name="New Staple Items" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="0" fullCalcOnLoad="1" iterateDelta="0.0001"/>
 </workbook>
 </file>
 
@@ -29,44 +28,54 @@
     </font>
     <font>
       <name val="Arial"/>
+      <family val="2"/>
       <b val="1"/>
-      <color rgb="00542916"/>
+      <color rgb="FF542916"/>
       <sz val="14"/>
     </font>
     <font>
       <name val="Arial"/>
-      <color rgb="002B241C"/>
+      <family val="2"/>
+      <color rgb="FF2B241C"/>
       <sz val="10"/>
     </font>
     <font>
       <name val="Arial"/>
-      <color rgb="002B241C"/>
+      <family val="2"/>
+      <color rgb="FF2B241C"/>
       <sz val="11"/>
     </font>
     <font>
       <name val="Arial"/>
+      <family val="2"/>
       <b val="1"/>
-      <color rgb="00542916"/>
+      <color rgb="FF542916"/>
       <sz val="11"/>
     </font>
     <font>
       <name val="Arial"/>
+      <family val="2"/>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
+      <color rgb="FFFFFFFF"/>
       <sz val="11"/>
     </font>
     <font>
       <name val="Arial"/>
+      <family val="2"/>
       <sz val="10"/>
     </font>
     <font>
       <name val="Arial"/>
+      <family val="2"/>
       <i val="1"/>
-      <color rgb="00808080"/>
+      <color rgb="FF808080"/>
       <sz val="10"/>
     </font>
     <font>
+      <name val="Calibri"/>
+      <family val="2"/>
       <b val="1"/>
+      <sz val="11"/>
     </font>
   </fonts>
   <fills count="4">
@@ -78,14 +87,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F2565C"/>
-        <bgColor rgb="00F2565C"/>
+        <fgColor rgb="FFF2565C"/>
+        <bgColor rgb="FFF2565C"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFF9C4"/>
-        <bgColor rgb="00FFF9C4"/>
+        <fgColor rgb="FFFFF9C4"/>
+        <bgColor rgb="FFFFF9C4"/>
       </patternFill>
     </fill>
   </fills>
@@ -99,17 +108,18 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="00D9D9D9"/>
+        <color rgb="FFD9D9D9"/>
       </left>
       <right style="thin">
-        <color rgb="00D9D9D9"/>
+        <color rgb="FFD9D9D9"/>
       </right>
       <top style="thin">
-        <color rgb="00D9D9D9"/>
+        <color rgb="FFD9D9D9"/>
       </top>
       <bottom style="thin">
-        <color rgb="00D9D9D9"/>
+        <color rgb="FFD9D9D9"/>
       </bottom>
+      <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
@@ -153,7 +163,7 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -542,7 +552,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:A52"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
   </cols>
@@ -555,7 +565,7 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr"/>
+      <c r="A2" s="2" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
@@ -579,7 +589,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="inlineStr"/>
+      <c r="A6" s="2" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
@@ -708,7 +718,7 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="2" t="inlineStr"/>
+      <c r="A25" s="2" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
@@ -732,7 +742,7 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="2" t="inlineStr"/>
+      <c r="A29" s="2" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="4" t="inlineStr">
@@ -798,7 +808,7 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="2" t="inlineStr"/>
+      <c r="A39" s="2" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="4" t="inlineStr">
@@ -896,7 +906,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:L119"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
@@ -906,9 +916,7 @@
     <col width="14" customWidth="1" min="6" max="6"/>
     <col width="22" customWidth="1" min="7" max="7"/>
     <col width="30" customWidth="1" min="8" max="8"/>
-    <col width="12" customWidth="1" min="9" max="9"/>
-    <col width="12" customWidth="1" min="10" max="10"/>
-    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="9" max="11"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -1382,6 +1390,11 @@
       <c r="K11" s="6" t="n">
         <v>7</v>
       </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>To-Go Yogurt</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="6" t="n">
@@ -1423,6 +1436,11 @@
       <c r="K12" s="6" t="n">
         <v>2</v>
       </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>To-Go Yogurt</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="6" t="n">
@@ -2047,6 +2065,11 @@
         <v>4</v>
       </c>
       <c r="K27" s="6" t="n"/>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>To-Go Snack</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="6" t="n">
@@ -2086,6 +2109,11 @@
         <v>4</v>
       </c>
       <c r="K28" s="6" t="n"/>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>To-Go Snack</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="6" t="n">
@@ -2125,6 +2153,11 @@
         <v>0</v>
       </c>
       <c r="K29" s="6" t="n"/>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>To-Go Snack</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="6" t="n">
@@ -5631,6 +5664,11 @@
         <v>0</v>
       </c>
       <c r="K117" s="6" t="n"/>
+      <c r="L117" t="inlineStr">
+        <is>
+          <t>To-Go Snack</t>
+        </is>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="6" t="n">
@@ -5712,7 +5750,7 @@
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="H2 H3 H4 H5 H6 H7 H8 H9 H10 H11 H12 H13 H14 H15 H16 H17 H18 H19 H20 H21 H22 H23 H24 H25 H26 H27 H28 H29 H30 H31 H32 H33 H34 H35 H36 H37 H38 H39 H40 H41 H42 H43 H44 H45 H46 H47 H48 H49 H50 H51 H52 H53 H54 H55 H56 H57 H58 H59 H60 H61 H62 H63 H64 H65 H66 H67 H68 H69 H70 H71 H72 H73 H74 H75 H76 H77 H78 H79 H80 H81 H82 H83 H84 H85 H86 H87 H88 H89 H90 H91 H92 H93 H94 H95 H96 H97 H98 H99 H100 H101 H102 H103 H104 H105 H106 H107 H108 H109 H110 H111 H112 H113 H114 H115 H116 H117 H118 H119" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Invalid brand" error="Choose yc, staple, or shared from the list." type="list">
+    <dataValidation sqref="H2:H119" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Invalid brand" error="Choose yc, staple, or shared from the list." type="list">
       <formula1>"yc,staple,shared"</formula1>
     </dataValidation>
   </dataValidations>
@@ -5728,7 +5766,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:H42"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
     <col width="34" customWidth="1" min="2" max="2"/>
@@ -5781,7 +5819,7 @@
         </is>
       </c>
     </row>
-    <row r="2">
+    <row r="2" ht="28" customHeight="1">
       <c r="A2" s="10" t="n">
         <v>1</v>
       </c>
@@ -5814,7 +5852,7 @@
         </is>
       </c>
     </row>
-    <row r="3">
+    <row r="3" ht="42" customHeight="1">
       <c r="A3" s="9" t="n">
         <v>2</v>
       </c>
@@ -5845,7 +5883,7 @@
         </is>
       </c>
     </row>
-    <row r="4">
+    <row r="4" ht="70" customHeight="1">
       <c r="A4" s="9" t="n">
         <v>3</v>
       </c>
@@ -5876,7 +5914,7 @@
         </is>
       </c>
     </row>
-    <row r="5">
+    <row r="5" ht="70" customHeight="1">
       <c r="A5" s="9" t="n">
         <v>4</v>
       </c>
@@ -5907,7 +5945,7 @@
         </is>
       </c>
     </row>
-    <row r="6">
+    <row r="6" ht="28" customHeight="1">
       <c r="A6" s="9" t="n">
         <v>5</v>
       </c>
@@ -5938,7 +5976,7 @@
         </is>
       </c>
     </row>
-    <row r="7">
+    <row r="7" ht="28" customHeight="1">
       <c r="A7" s="9" t="n">
         <v>6</v>
       </c>
@@ -5973,10 +6011,26 @@
       <c r="A8" s="9" t="n">
         <v>7</v>
       </c>
-      <c r="B8" s="8" t="n"/>
-      <c r="C8" s="8" t="n"/>
-      <c r="D8" s="8" t="n"/>
-      <c r="E8" s="8" t="n"/>
+      <c r="B8" s="8" t="inlineStr">
+        <is>
+          <t>Feta Cheese</t>
+        </is>
+      </c>
+      <c r="C8" s="8" t="inlineStr">
+        <is>
+          <t>To-Go Cheese</t>
+        </is>
+      </c>
+      <c r="D8" s="8" t="inlineStr">
+        <is>
+          <t>กระปุก</t>
+        </is>
+      </c>
+      <c r="E8" s="8" t="inlineStr">
+        <is>
+          <t>shared</t>
+        </is>
+      </c>
       <c r="F8" s="9" t="n"/>
       <c r="G8" s="8" t="n"/>
     </row>
@@ -5984,10 +6038,26 @@
       <c r="A9" s="9" t="n">
         <v>8</v>
       </c>
-      <c r="B9" s="8" t="n"/>
-      <c r="C9" s="8" t="n"/>
-      <c r="D9" s="8" t="n"/>
-      <c r="E9" s="8" t="n"/>
+      <c r="B9" s="8" t="inlineStr">
+        <is>
+          <t>Ricotta</t>
+        </is>
+      </c>
+      <c r="C9" s="8" t="inlineStr">
+        <is>
+          <t>To-Go Cheese</t>
+        </is>
+      </c>
+      <c r="D9" s="8" t="inlineStr">
+        <is>
+          <t>กระปุก</t>
+        </is>
+      </c>
+      <c r="E9" s="8" t="inlineStr">
+        <is>
+          <t>shared</t>
+        </is>
+      </c>
       <c r="F9" s="9" t="n"/>
       <c r="G9" s="8" t="n"/>
     </row>
@@ -5995,10 +6065,26 @@
       <c r="A10" s="9" t="n">
         <v>9</v>
       </c>
-      <c r="B10" s="8" t="n"/>
-      <c r="C10" s="8" t="n"/>
-      <c r="D10" s="8" t="n"/>
-      <c r="E10" s="8" t="n"/>
+      <c r="B10" s="8" t="inlineStr">
+        <is>
+          <t>Ham Cheese Sandwich</t>
+        </is>
+      </c>
+      <c r="C10" s="8" t="inlineStr">
+        <is>
+          <t>To-Go Sandwich &amp; Salad</t>
+        </is>
+      </c>
+      <c r="D10" s="8" t="inlineStr">
+        <is>
+          <t>ชิ้น</t>
+        </is>
+      </c>
+      <c r="E10" s="8" t="inlineStr">
+        <is>
+          <t>shared</t>
+        </is>
+      </c>
       <c r="F10" s="9" t="n"/>
       <c r="G10" s="8" t="n"/>
     </row>
@@ -6006,10 +6092,26 @@
       <c r="A11" s="9" t="n">
         <v>10</v>
       </c>
-      <c r="B11" s="8" t="n"/>
-      <c r="C11" s="8" t="n"/>
-      <c r="D11" s="8" t="n"/>
-      <c r="E11" s="8" t="n"/>
+      <c r="B11" s="8" t="inlineStr">
+        <is>
+          <t>Egg Salad Sandwich</t>
+        </is>
+      </c>
+      <c r="C11" s="8" t="inlineStr">
+        <is>
+          <t>To-Go Sandwich &amp; Salad</t>
+        </is>
+      </c>
+      <c r="D11" s="8" t="inlineStr">
+        <is>
+          <t>ชิ้น</t>
+        </is>
+      </c>
+      <c r="E11" s="8" t="inlineStr">
+        <is>
+          <t>shared</t>
+        </is>
+      </c>
       <c r="F11" s="9" t="n"/>
       <c r="G11" s="8" t="n"/>
     </row>
@@ -6017,10 +6119,26 @@
       <c r="A12" s="9" t="n">
         <v>11</v>
       </c>
-      <c r="B12" s="8" t="n"/>
-      <c r="C12" s="8" t="n"/>
-      <c r="D12" s="8" t="n"/>
-      <c r="E12" s="8" t="n"/>
+      <c r="B12" s="8" t="inlineStr">
+        <is>
+          <t>Tuna Sandwich</t>
+        </is>
+      </c>
+      <c r="C12" s="8" t="inlineStr">
+        <is>
+          <t>To-Go Sandwich &amp; Salad</t>
+        </is>
+      </c>
+      <c r="D12" s="8" t="inlineStr">
+        <is>
+          <t>ชิ้น</t>
+        </is>
+      </c>
+      <c r="E12" s="8" t="inlineStr">
+        <is>
+          <t>shared</t>
+        </is>
+      </c>
       <c r="F12" s="9" t="n"/>
       <c r="G12" s="8" t="n"/>
     </row>
@@ -6028,10 +6146,26 @@
       <c r="A13" s="9" t="n">
         <v>12</v>
       </c>
-      <c r="B13" s="8" t="n"/>
-      <c r="C13" s="8" t="n"/>
-      <c r="D13" s="8" t="n"/>
-      <c r="E13" s="8" t="n"/>
+      <c r="B13" s="8" t="inlineStr">
+        <is>
+          <t>Sour Hour - Ginger Lemon</t>
+        </is>
+      </c>
+      <c r="C13" s="8" t="inlineStr">
+        <is>
+          <t>To-Go Beverage</t>
+        </is>
+      </c>
+      <c r="D13" s="8" t="inlineStr">
+        <is>
+          <t>กระป๋อง</t>
+        </is>
+      </c>
+      <c r="E13" s="8" t="inlineStr">
+        <is>
+          <t>shared</t>
+        </is>
+      </c>
       <c r="F13" s="9" t="n"/>
       <c r="G13" s="8" t="n"/>
     </row>
@@ -6039,10 +6173,26 @@
       <c r="A14" s="9" t="n">
         <v>13</v>
       </c>
-      <c r="B14" s="8" t="n"/>
-      <c r="C14" s="8" t="n"/>
-      <c r="D14" s="8" t="n"/>
-      <c r="E14" s="8" t="n"/>
+      <c r="B14" s="8" t="inlineStr">
+        <is>
+          <t>Sour Hour - Peach Lychee</t>
+        </is>
+      </c>
+      <c r="C14" s="8" t="inlineStr">
+        <is>
+          <t>To-Go Beverage</t>
+        </is>
+      </c>
+      <c r="D14" s="8" t="inlineStr">
+        <is>
+          <t>กระป๋อง</t>
+        </is>
+      </c>
+      <c r="E14" s="8" t="inlineStr">
+        <is>
+          <t>shared</t>
+        </is>
+      </c>
       <c r="F14" s="9" t="n"/>
       <c r="G14" s="8" t="n"/>
     </row>
@@ -6050,10 +6200,26 @@
       <c r="A15" s="9" t="n">
         <v>14</v>
       </c>
-      <c r="B15" s="8" t="n"/>
-      <c r="C15" s="8" t="n"/>
-      <c r="D15" s="8" t="n"/>
-      <c r="E15" s="8" t="n"/>
+      <c r="B15" s="8" t="inlineStr">
+        <is>
+          <t>San Pellegrino</t>
+        </is>
+      </c>
+      <c r="C15" s="8" t="inlineStr">
+        <is>
+          <t>To-Go Beverage</t>
+        </is>
+      </c>
+      <c r="D15" s="8" t="inlineStr">
+        <is>
+          <t>ขวด</t>
+        </is>
+      </c>
+      <c r="E15" s="8" t="inlineStr">
+        <is>
+          <t>shared</t>
+        </is>
+      </c>
       <c r="F15" s="9" t="n"/>
       <c r="G15" s="8" t="n"/>
     </row>
@@ -6061,10 +6227,26 @@
       <c r="A16" s="9" t="n">
         <v>15</v>
       </c>
-      <c r="B16" s="8" t="n"/>
-      <c r="C16" s="8" t="n"/>
-      <c r="D16" s="8" t="n"/>
-      <c r="E16" s="8" t="n"/>
+      <c r="B16" s="8" t="inlineStr">
+        <is>
+          <t>Coca Cola</t>
+        </is>
+      </c>
+      <c r="C16" s="8" t="inlineStr">
+        <is>
+          <t>To-Go Beverage</t>
+        </is>
+      </c>
+      <c r="D16" s="8" t="inlineStr">
+        <is>
+          <t>กระป๋อง</t>
+        </is>
+      </c>
+      <c r="E16" s="8" t="inlineStr">
+        <is>
+          <t>shared</t>
+        </is>
+      </c>
       <c r="F16" s="9" t="n"/>
       <c r="G16" s="8" t="n"/>
     </row>
@@ -6072,10 +6254,26 @@
       <c r="A17" s="9" t="n">
         <v>16</v>
       </c>
-      <c r="B17" s="8" t="n"/>
-      <c r="C17" s="8" t="n"/>
-      <c r="D17" s="8" t="n"/>
-      <c r="E17" s="8" t="n"/>
+      <c r="B17" s="8" t="inlineStr">
+        <is>
+          <t>Sprite</t>
+        </is>
+      </c>
+      <c r="C17" s="8" t="inlineStr">
+        <is>
+          <t>To-Go Beverage</t>
+        </is>
+      </c>
+      <c r="D17" s="8" t="inlineStr">
+        <is>
+          <t>กระป๋อง</t>
+        </is>
+      </c>
+      <c r="E17" s="8" t="inlineStr">
+        <is>
+          <t>shared</t>
+        </is>
+      </c>
       <c r="F17" s="9" t="n"/>
       <c r="G17" s="8" t="n"/>
     </row>

</xml_diff>

<commit_message>
NCD_Brand_Tagging: อัปเดตชื่อรายการ + เพิ่ม To-Go Salad/Overnight Oats/Chia Pudding (backup)
ผมไม่ได้แตะ/regenerate ใดๆ แค่ commit เก็บสถานะไว้กันหาย
- แก้ชื่อ sandwich/wrap เป็นชื่อจริง (Chicken Caesar Wrap, Chicken Pesto Wrap, Tuna eggs and cheese wrap)
- แก้ชื่อ Yogurt Bowl 1-3 เป็นชื่อจริง (Apple pecan pie / PB&J / Blueberry pie greek yogurt)
- เพิ่มรายการใหม่ 6 รายการ (แถว 83-88): Chicken Waldorf Salad, Tuna Herb Salad, Chicken Caesar Salad
  (To-Go Sandwich & Salad), Biscoff overnight oats, Dark Chocolate Chia Pudding, Honey Yogurt Chia Pudding
  (To-Go Overnight Oats / To-Go Chia Pudding)
- รวมตอนนี้มี New Staple Items ทั้งหมด 91 แถว (No. 1-89)
</commit_message>
<xml_diff>
--- a/NCD_Brand_Tagging.xlsx
+++ b/NCD_Brand_Tagging.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10802"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10810"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/praee/Desktop/CLAUDE/BQMP OPS/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4BE1FCAC-729F-DD4D-A549-DBACF1DFBFF4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{81166571-3007-AC4C-B29A-6EFA991AC35E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="17220" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -17,7 +17,20 @@
     <sheet name="Existing Items" sheetId="2" r:id="rId2"/>
     <sheet name="New Staple Items" sheetId="3" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="0" iterateDelta="1E-4"/>
+  <calcPr calcId="191029" iterateDelta="1E-4"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -74,7 +87,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1041" uniqueCount="502">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1068" uniqueCount="510">
   <si>
     <t>No.</t>
   </si>
@@ -1255,21 +1268,12 @@
     <t>Ricotta</t>
   </si>
   <si>
-    <t>Ham Cheese Sandwich</t>
-  </si>
-  <si>
     <t>To-Go Sandwich &amp; Salad</t>
   </si>
   <si>
     <t>ชิ้น</t>
   </si>
   <si>
-    <t>Egg Salad Sandwich</t>
-  </si>
-  <si>
-    <t>Tuna Sandwich</t>
-  </si>
-  <si>
     <t>Sour Hour - Ginger Lemon</t>
   </si>
   <si>
@@ -1402,15 +1406,6 @@
     <t>Orange Juice</t>
   </si>
   <si>
-    <t>Yogurt Bowl 1</t>
-  </si>
-  <si>
-    <t>Yogurt Bowl 2</t>
-  </si>
-  <si>
-    <t>Yogurt Bowl 3</t>
-  </si>
-  <si>
     <t>Plastic Wrap</t>
   </si>
   <si>
@@ -1580,13 +1575,55 @@
   </si>
   <si>
     <t>Chocolate Fudge Drink</t>
+  </si>
+  <si>
+    <t>Chicken Caesar Wrap</t>
+  </si>
+  <si>
+    <t>Chicken Pesto Wrap</t>
+  </si>
+  <si>
+    <t>Tuna  eggs and cheese wrap</t>
+  </si>
+  <si>
+    <t>Chicken Waldorf Salad</t>
+  </si>
+  <si>
+    <t>Chicken Caesar Salad</t>
+  </si>
+  <si>
+    <t>Tuna Herb Salad</t>
+  </si>
+  <si>
+    <t>Apple pecan pie greek yogurt</t>
+  </si>
+  <si>
+    <t>PB&amp;J greek yogurt</t>
+  </si>
+  <si>
+    <t>Blueberry pie greek yogurt</t>
+  </si>
+  <si>
+    <t>Biscoff overnight oats</t>
+  </si>
+  <si>
+    <t>To-Go Overnight Oats</t>
+  </si>
+  <si>
+    <t>Dark Chocolate Chia Pudding</t>
+  </si>
+  <si>
+    <t>Honey Yogurt Chia Pudding</t>
+  </si>
+  <si>
+    <t>To-Go Chia Pudding</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="11" x14ac:knownFonts="1">
+  <fonts count="12">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1656,6 +1693,11 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="YAHOUAhS5u0_0"/>
     </font>
   </fonts>
   <fills count="4">
@@ -1801,9 +1843,7 @@
     <xf numFmtId="0" fontId="6" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2107,272 +2147,272 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:A57"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="100" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" ht="22" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:1" ht="22" customHeight="1">
       <c r="A1" s="1" t="s">
         <v>321</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:1">
       <c r="A2" s="2"/>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:1">
       <c r="A3" s="3" t="s">
         <v>322</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:1">
       <c r="A4" s="3" t="s">
         <v>323</v>
       </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:1">
       <c r="A5" s="3" t="s">
         <v>324</v>
       </c>
     </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:1">
       <c r="A6" s="2"/>
     </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:1">
       <c r="A7" s="4" t="s">
         <v>325</v>
       </c>
     </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:1">
       <c r="A8" s="3" t="s">
         <v>326</v>
       </c>
     </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:1">
       <c r="A9" s="3" t="s">
         <v>327</v>
       </c>
     </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:1">
       <c r="A10" s="3" t="s">
         <v>328</v>
       </c>
     </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:1">
       <c r="A11" s="3" t="s">
         <v>329</v>
       </c>
     </row>
-    <row r="12" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:1">
       <c r="A12" s="3" t="s">
         <v>330</v>
       </c>
     </row>
-    <row r="13" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:1">
       <c r="A13" s="3" t="s">
         <v>331</v>
       </c>
     </row>
-    <row r="14" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:1">
       <c r="A14" s="3" t="s">
         <v>332</v>
       </c>
     </row>
-    <row r="15" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:1">
       <c r="A15" s="3" t="s">
         <v>333</v>
       </c>
     </row>
-    <row r="16" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:1">
       <c r="A16" s="3" t="s">
         <v>334</v>
       </c>
     </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:1">
       <c r="A17" s="3" t="s">
         <v>335</v>
       </c>
     </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:1">
       <c r="A18" s="3" t="s">
         <v>336</v>
       </c>
     </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:1">
       <c r="A19" s="3" t="s">
         <v>337</v>
       </c>
     </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:1">
       <c r="A20" s="3" t="s">
         <v>338</v>
       </c>
     </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:1">
       <c r="A21" s="3" t="s">
         <v>339</v>
       </c>
     </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:1">
       <c r="A22" s="3" t="s">
         <v>340</v>
       </c>
     </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:1">
       <c r="A23" s="3" t="s">
         <v>341</v>
       </c>
     </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:1">
       <c r="A24" s="3" t="s">
         <v>342</v>
       </c>
     </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:1">
       <c r="A25" s="2"/>
     </row>
-    <row r="26" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:1">
       <c r="A26" s="3" t="s">
         <v>343</v>
       </c>
     </row>
-    <row r="27" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:1">
       <c r="A27" s="3" t="s">
         <v>344</v>
       </c>
     </row>
-    <row r="28" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:1">
       <c r="A28" s="3" t="s">
         <v>345</v>
       </c>
     </row>
-    <row r="29" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:1">
       <c r="A29" s="2"/>
     </row>
-    <row r="30" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:1">
       <c r="A30" s="4" t="s">
         <v>346</v>
       </c>
     </row>
-    <row r="31" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:1">
       <c r="A31" s="3" t="s">
         <v>347</v>
       </c>
     </row>
-    <row r="32" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:1">
       <c r="A32" s="3" t="s">
         <v>348</v>
       </c>
     </row>
-    <row r="33" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:1">
       <c r="A33" s="3" t="s">
         <v>349</v>
       </c>
     </row>
-    <row r="34" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:1">
       <c r="A34" s="3" t="s">
         <v>350</v>
       </c>
     </row>
-    <row r="35" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:1">
       <c r="A35" s="3" t="s">
         <v>351</v>
       </c>
     </row>
-    <row r="36" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:1">
       <c r="A36" s="3" t="s">
         <v>352</v>
       </c>
     </row>
-    <row r="37" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:1">
       <c r="A37" s="3" t="s">
         <v>353</v>
       </c>
     </row>
-    <row r="38" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:1">
       <c r="A38" s="3" t="s">
         <v>354</v>
       </c>
     </row>
-    <row r="39" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:1">
       <c r="A39" s="2"/>
     </row>
-    <row r="40" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:1">
       <c r="A40" s="4" t="s">
         <v>355</v>
       </c>
     </row>
-    <row r="42" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:1">
       <c r="A42" t="s">
         <v>356</v>
       </c>
     </row>
-    <row r="43" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:1">
       <c r="A43" t="s">
         <v>357</v>
       </c>
     </row>
-    <row r="44" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:1">
       <c r="A44" t="s">
         <v>358</v>
       </c>
     </row>
-    <row r="45" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:1">
       <c r="A45" t="s">
         <v>359</v>
       </c>
     </row>
-    <row r="46" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:1">
       <c r="A46" t="s">
         <v>360</v>
       </c>
     </row>
-    <row r="47" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:1">
       <c r="A47" t="s">
         <v>361</v>
       </c>
     </row>
-    <row r="48" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:1">
       <c r="A48" t="s">
         <v>362</v>
       </c>
     </row>
-    <row r="49" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:1">
       <c r="A49" t="s">
         <v>363</v>
       </c>
     </row>
-    <row r="50" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:1">
       <c r="A50" t="s">
         <v>364</v>
       </c>
     </row>
-    <row r="51" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:1">
       <c r="A51" t="s">
         <v>365</v>
       </c>
     </row>
-    <row r="52" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:1">
       <c r="A52" t="s">
         <v>366</v>
       </c>
     </row>
-    <row r="54" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:1">
       <c r="A54" t="s">
         <v>367</v>
       </c>
     </row>
-    <row r="55" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:1">
       <c r="A55" t="s">
         <v>368</v>
       </c>
     </row>
-    <row r="56" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:1">
       <c r="A56" t="s">
         <v>369</v>
       </c>
     </row>
-    <row r="57" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:1">
       <c r="A57" t="s">
         <v>370</v>
       </c>
@@ -2385,7 +2425,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:M119"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
     <col min="2" max="2" width="10" customWidth="1"/>
@@ -2398,7 +2438,7 @@
     <col min="9" max="11" width="12" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:13" ht="30" customHeight="1">
       <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
@@ -2439,7 +2479,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:13">
       <c r="A2" s="6">
         <v>1</v>
       </c>
@@ -2472,7 +2512,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:13">
       <c r="A3" s="6">
         <v>2</v>
       </c>
@@ -2486,7 +2526,7 @@
         <v>19</v>
       </c>
       <c r="E3" s="8" t="s">
-        <v>409</v>
+        <v>406</v>
       </c>
       <c r="F3" s="7" t="s">
         <v>16</v>
@@ -2507,7 +2547,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:13">
       <c r="A4" s="6">
         <v>3</v>
       </c>
@@ -2538,7 +2578,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:13">
       <c r="A5" s="6">
         <v>4</v>
       </c>
@@ -2569,7 +2609,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:13">
       <c r="A6" s="6">
         <v>5</v>
       </c>
@@ -2600,7 +2640,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:13">
       <c r="A7" s="6">
         <v>6</v>
       </c>
@@ -2631,7 +2671,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:13">
       <c r="A8" s="6">
         <v>7</v>
       </c>
@@ -2662,7 +2702,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:13">
       <c r="A9" s="6">
         <v>8</v>
       </c>
@@ -2693,7 +2733,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:13">
       <c r="A10" s="6">
         <v>9</v>
       </c>
@@ -2724,7 +2764,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:13">
       <c r="A11" s="6">
         <v>10</v>
       </c>
@@ -2760,7 +2800,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:13">
       <c r="A12" s="6">
         <v>11</v>
       </c>
@@ -2796,7 +2836,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:13">
       <c r="A13" s="6">
         <v>12</v>
       </c>
@@ -2825,7 +2865,7 @@
       </c>
       <c r="K13" s="6"/>
     </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:13">
       <c r="A14" s="6">
         <v>13</v>
       </c>
@@ -2854,7 +2894,7 @@
       </c>
       <c r="K14" s="6"/>
     </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:13">
       <c r="A15" s="6">
         <v>14</v>
       </c>
@@ -2881,7 +2921,7 @@
       <c r="J15" s="6"/>
       <c r="K15" s="6"/>
     </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:13">
       <c r="A16" s="6">
         <v>15</v>
       </c>
@@ -2908,7 +2948,7 @@
       <c r="J16" s="6"/>
       <c r="K16" s="6"/>
     </row>
-    <row r="17" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:12">
       <c r="A17" s="6">
         <v>16</v>
       </c>
@@ -2937,7 +2977,7 @@
       </c>
       <c r="K17" s="6"/>
     </row>
-    <row r="18" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:12">
       <c r="A18" s="6">
         <v>17</v>
       </c>
@@ -2951,7 +2991,7 @@
         <v>60</v>
       </c>
       <c r="E18" s="8" t="s">
-        <v>408</v>
+        <v>405</v>
       </c>
       <c r="F18" s="7" t="s">
         <v>57</v>
@@ -2970,7 +3010,7 @@
       </c>
       <c r="K18" s="6"/>
     </row>
-    <row r="19" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:12">
       <c r="A19" s="6">
         <v>18</v>
       </c>
@@ -2995,7 +3035,7 @@
       <c r="J19" s="6"/>
       <c r="K19" s="6"/>
     </row>
-    <row r="20" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:12">
       <c r="A20" s="6">
         <v>19</v>
       </c>
@@ -3009,7 +3049,7 @@
         <v>66</v>
       </c>
       <c r="E20" s="8" t="s">
-        <v>407</v>
+        <v>404</v>
       </c>
       <c r="F20" s="7" t="s">
         <v>67</v>
@@ -3031,7 +3071,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="21" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:12">
       <c r="A21" s="6">
         <v>20</v>
       </c>
@@ -3045,7 +3085,7 @@
         <v>71</v>
       </c>
       <c r="E21" s="8" t="s">
-        <v>410</v>
+        <v>407</v>
       </c>
       <c r="F21" s="7" t="s">
         <v>72</v>
@@ -3069,7 +3109,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="22" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:12">
       <c r="A22" s="6">
         <v>21</v>
       </c>
@@ -3083,7 +3123,7 @@
         <v>74</v>
       </c>
       <c r="E22" s="8" t="s">
-        <v>411</v>
+        <v>408</v>
       </c>
       <c r="F22" s="7" t="s">
         <v>72</v>
@@ -3107,7 +3147,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="23" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:12">
       <c r="A23" s="6">
         <v>22</v>
       </c>
@@ -3121,7 +3161,7 @@
         <v>76</v>
       </c>
       <c r="E23" s="8" t="s">
-        <v>412</v>
+        <v>409</v>
       </c>
       <c r="F23" s="7" t="s">
         <v>72</v>
@@ -3145,7 +3185,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="24" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:12">
       <c r="A24" s="6">
         <v>23</v>
       </c>
@@ -3159,7 +3199,7 @@
         <v>78</v>
       </c>
       <c r="E24" s="8" t="s">
-        <v>413</v>
+        <v>410</v>
       </c>
       <c r="F24" s="7" t="s">
         <v>72</v>
@@ -3183,7 +3223,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="25" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:12">
       <c r="A25" s="6">
         <v>24</v>
       </c>
@@ -3197,7 +3237,7 @@
         <v>80</v>
       </c>
       <c r="E25" s="8" t="s">
-        <v>414</v>
+        <v>411</v>
       </c>
       <c r="F25" s="7" t="s">
         <v>72</v>
@@ -3221,7 +3261,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="26" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:12">
       <c r="A26" s="6">
         <v>25</v>
       </c>
@@ -3235,7 +3275,7 @@
         <v>82</v>
       </c>
       <c r="E26" s="8" t="s">
-        <v>415</v>
+        <v>412</v>
       </c>
       <c r="F26" s="7" t="s">
         <v>72</v>
@@ -3259,7 +3299,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="27" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:12">
       <c r="A27" s="6">
         <v>26</v>
       </c>
@@ -3273,7 +3313,7 @@
         <v>85</v>
       </c>
       <c r="E27" s="8" t="s">
-        <v>417</v>
+        <v>414</v>
       </c>
       <c r="F27" s="7" t="s">
         <v>64</v>
@@ -3295,7 +3335,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="28" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:12">
       <c r="A28" s="6">
         <v>27</v>
       </c>
@@ -3309,7 +3349,7 @@
         <v>89</v>
       </c>
       <c r="E28" s="8" t="s">
-        <v>416</v>
+        <v>413</v>
       </c>
       <c r="F28" s="7" t="s">
         <v>64</v>
@@ -3331,7 +3371,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="29" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:12">
       <c r="A29" s="6">
         <v>28</v>
       </c>
@@ -3365,7 +3405,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="30" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:12">
       <c r="A30" s="6">
         <v>29</v>
       </c>
@@ -3398,7 +3438,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:12">
       <c r="A31" s="6">
         <v>30</v>
       </c>
@@ -3431,7 +3471,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="32" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:12">
       <c r="A32" s="6">
         <v>31</v>
       </c>
@@ -3464,7 +3504,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="33" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:11">
       <c r="A33" s="6">
         <v>32</v>
       </c>
@@ -3497,7 +3537,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:11">
       <c r="A34" s="6">
         <v>33</v>
       </c>
@@ -3530,7 +3570,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="35" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:11">
       <c r="A35" s="6">
         <v>34</v>
       </c>
@@ -3561,7 +3601,7 @@
       </c>
       <c r="K35" s="6"/>
     </row>
-    <row r="36" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:11">
       <c r="A36" s="6">
         <v>35</v>
       </c>
@@ -3592,7 +3632,7 @@
       </c>
       <c r="K36" s="6"/>
     </row>
-    <row r="37" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:11">
       <c r="A37" s="6">
         <v>36</v>
       </c>
@@ -3623,7 +3663,7 @@
       </c>
       <c r="K37" s="6"/>
     </row>
-    <row r="38" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:11">
       <c r="A38" s="6">
         <v>37</v>
       </c>
@@ -3654,7 +3694,7 @@
       </c>
       <c r="K38" s="6"/>
     </row>
-    <row r="39" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:11">
       <c r="A39" s="6">
         <v>38</v>
       </c>
@@ -3687,7 +3727,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="40" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:11">
       <c r="A40" s="6">
         <v>39</v>
       </c>
@@ -3720,7 +3760,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="41" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:11">
       <c r="A41" s="6">
         <v>40</v>
       </c>
@@ -3753,7 +3793,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="42" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:11">
       <c r="A42" s="6">
         <v>41</v>
       </c>
@@ -3784,7 +3824,7 @@
       </c>
       <c r="K42" s="6"/>
     </row>
-    <row r="43" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:11">
       <c r="A43" s="6">
         <v>42</v>
       </c>
@@ -3815,7 +3855,7 @@
       </c>
       <c r="K43" s="6"/>
     </row>
-    <row r="44" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:11">
       <c r="A44" s="6">
         <v>43</v>
       </c>
@@ -3848,7 +3888,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:11">
       <c r="A45" s="6">
         <v>44</v>
       </c>
@@ -3873,7 +3913,7 @@
       <c r="J45" s="6"/>
       <c r="K45" s="6"/>
     </row>
-    <row r="46" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:11">
       <c r="A46" s="6">
         <v>45</v>
       </c>
@@ -3898,7 +3938,7 @@
       <c r="J46" s="6"/>
       <c r="K46" s="6"/>
     </row>
-    <row r="47" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:11">
       <c r="A47" s="6">
         <v>46</v>
       </c>
@@ -3931,7 +3971,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="48" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:11">
       <c r="A48" s="6">
         <v>47</v>
       </c>
@@ -3956,7 +3996,7 @@
       <c r="J48" s="6"/>
       <c r="K48" s="6"/>
     </row>
-    <row r="49" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:11">
       <c r="A49" s="6">
         <v>48</v>
       </c>
@@ -3989,7 +4029,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="50" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:11">
       <c r="A50" s="6">
         <v>49</v>
       </c>
@@ -4022,7 +4062,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="51" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:11">
       <c r="A51" s="6">
         <v>50</v>
       </c>
@@ -4055,7 +4095,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="52" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:11">
       <c r="A52" s="6">
         <v>51</v>
       </c>
@@ -4088,7 +4128,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="53" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:11">
       <c r="A53" s="6">
         <v>52</v>
       </c>
@@ -4102,7 +4142,7 @@
         <v>157</v>
       </c>
       <c r="E53" s="7" t="s">
-        <v>428</v>
+        <v>425</v>
       </c>
       <c r="F53" s="7" t="s">
         <v>126</v>
@@ -4123,7 +4163,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="54" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:11">
       <c r="A54" s="6">
         <v>53</v>
       </c>
@@ -4154,7 +4194,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="55" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:11">
       <c r="A55" s="6">
         <v>54</v>
       </c>
@@ -4185,7 +4225,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="56" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:11">
       <c r="A56" s="6">
         <v>55</v>
       </c>
@@ -4199,7 +4239,7 @@
         <v>165</v>
       </c>
       <c r="E56" s="8" t="s">
-        <v>418</v>
+        <v>415</v>
       </c>
       <c r="F56" s="7" t="s">
         <v>161</v>
@@ -4220,7 +4260,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="57" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:11">
       <c r="A57" s="6">
         <v>56</v>
       </c>
@@ -4255,7 +4295,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="58" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:11">
       <c r="A58" s="6">
         <v>57</v>
       </c>
@@ -4269,7 +4309,7 @@
         <v>171</v>
       </c>
       <c r="E58" s="8" t="s">
-        <v>424</v>
+        <v>421</v>
       </c>
       <c r="F58" s="7" t="s">
         <v>161</v>
@@ -4290,7 +4330,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="59" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:11">
       <c r="A59" s="6">
         <v>58</v>
       </c>
@@ -4304,7 +4344,7 @@
         <v>173</v>
       </c>
       <c r="E59" s="8" t="s">
-        <v>425</v>
+        <v>422</v>
       </c>
       <c r="F59" s="7" t="s">
         <v>161</v>
@@ -4325,7 +4365,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="60" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:11">
       <c r="A60" s="6">
         <v>59</v>
       </c>
@@ -4339,7 +4379,7 @@
         <v>175</v>
       </c>
       <c r="E60" s="8" t="s">
-        <v>426</v>
+        <v>423</v>
       </c>
       <c r="F60" s="7" t="s">
         <v>161</v>
@@ -4360,7 +4400,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="61" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:11">
       <c r="A61" s="6">
         <v>60</v>
       </c>
@@ -4393,7 +4433,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="62" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:11">
       <c r="A62" s="6">
         <v>61</v>
       </c>
@@ -4407,7 +4447,7 @@
         <v>180</v>
       </c>
       <c r="E62" s="7" t="s">
-        <v>427</v>
+        <v>424</v>
       </c>
       <c r="F62" s="7" t="s">
         <v>161</v>
@@ -4428,7 +4468,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="63" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:11">
       <c r="A63" s="6">
         <v>62</v>
       </c>
@@ -4459,7 +4499,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="64" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:11">
       <c r="A64" s="6">
         <v>63</v>
       </c>
@@ -4473,7 +4513,7 @@
         <v>184</v>
       </c>
       <c r="E64" s="8" t="s">
-        <v>423</v>
+        <v>420</v>
       </c>
       <c r="F64" s="7" t="s">
         <v>161</v>
@@ -4494,7 +4534,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="65" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:11">
       <c r="A65" s="6">
         <v>64</v>
       </c>
@@ -4527,7 +4567,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="66" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="66" spans="1:11">
       <c r="A66" s="6">
         <v>65</v>
       </c>
@@ -4560,7 +4600,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="67" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:11">
       <c r="A67" s="6">
         <v>66</v>
       </c>
@@ -4593,7 +4633,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="68" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="68" spans="1:11">
       <c r="A68" s="6">
         <v>67</v>
       </c>
@@ -4626,7 +4666,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="69" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="69" spans="1:11">
       <c r="A69" s="6">
         <v>68</v>
       </c>
@@ -4659,7 +4699,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="70" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="70" spans="1:11">
       <c r="A70" s="6">
         <v>69</v>
       </c>
@@ -4690,7 +4730,7 @@
       </c>
       <c r="K70" s="6"/>
     </row>
-    <row r="71" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="71" spans="1:11">
       <c r="A71" s="6">
         <v>70</v>
       </c>
@@ -4723,7 +4763,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="72" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="72" spans="1:11">
       <c r="A72" s="6">
         <v>71</v>
       </c>
@@ -4754,7 +4794,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="73" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="73" spans="1:11">
       <c r="A73" s="6">
         <v>72</v>
       </c>
@@ -4785,7 +4825,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="74" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="74" spans="1:11">
       <c r="A74" s="6">
         <v>73</v>
       </c>
@@ -4816,7 +4856,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="75" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="75" spans="1:11">
       <c r="A75" s="6">
         <v>74</v>
       </c>
@@ -4847,7 +4887,7 @@
       </c>
       <c r="K75" s="6"/>
     </row>
-    <row r="76" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="76" spans="1:11">
       <c r="A76" s="6">
         <v>75</v>
       </c>
@@ -4880,7 +4920,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="77" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="77" spans="1:11">
       <c r="A77" s="6">
         <v>76</v>
       </c>
@@ -4913,7 +4953,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="78" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="78" spans="1:11">
       <c r="A78" s="6">
         <v>77</v>
       </c>
@@ -4946,7 +4986,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="79" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="79" spans="1:11">
       <c r="A79" s="6">
         <v>78</v>
       </c>
@@ -4979,7 +5019,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="80" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="80" spans="1:11">
       <c r="A80" s="6">
         <v>79</v>
       </c>
@@ -5008,7 +5048,7 @@
       </c>
       <c r="K80" s="6"/>
     </row>
-    <row r="81" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="81" spans="1:11">
       <c r="A81" s="6">
         <v>80</v>
       </c>
@@ -5037,7 +5077,7 @@
       </c>
       <c r="K81" s="6"/>
     </row>
-    <row r="82" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="82" spans="1:11">
       <c r="A82" s="6">
         <v>81</v>
       </c>
@@ -5066,7 +5106,7 @@
       </c>
       <c r="K82" s="6"/>
     </row>
-    <row r="83" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="83" spans="1:11">
       <c r="A83" s="6">
         <v>82</v>
       </c>
@@ -5095,7 +5135,7 @@
       </c>
       <c r="K83" s="6"/>
     </row>
-    <row r="84" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="84" spans="1:11">
       <c r="A84" s="6">
         <v>83</v>
       </c>
@@ -5126,7 +5166,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="85" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="85" spans="1:11">
       <c r="A85" s="6">
         <v>84</v>
       </c>
@@ -5155,7 +5195,7 @@
       </c>
       <c r="K85" s="6"/>
     </row>
-    <row r="86" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="86" spans="1:11">
       <c r="A86" s="6">
         <v>85</v>
       </c>
@@ -5188,7 +5228,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="87" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="87" spans="1:11">
       <c r="A87" s="6">
         <v>86</v>
       </c>
@@ -5219,7 +5259,7 @@
       </c>
       <c r="K87" s="6"/>
     </row>
-    <row r="88" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="88" spans="1:11">
       <c r="A88" s="6">
         <v>87</v>
       </c>
@@ -5250,7 +5290,7 @@
       </c>
       <c r="K88" s="6"/>
     </row>
-    <row r="89" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="89" spans="1:11">
       <c r="A89" s="6">
         <v>88</v>
       </c>
@@ -5279,7 +5319,7 @@
       </c>
       <c r="K89" s="6"/>
     </row>
-    <row r="90" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="90" spans="1:11">
       <c r="A90" s="6">
         <v>89</v>
       </c>
@@ -5310,7 +5350,7 @@
       </c>
       <c r="K90" s="6"/>
     </row>
-    <row r="91" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="91" spans="1:11">
       <c r="A91" s="6">
         <v>90</v>
       </c>
@@ -5339,7 +5379,7 @@
       <c r="J91" s="6"/>
       <c r="K91" s="6"/>
     </row>
-    <row r="92" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="92" spans="1:11">
       <c r="A92" s="6">
         <v>91</v>
       </c>
@@ -5370,7 +5410,7 @@
       </c>
       <c r="K92" s="6"/>
     </row>
-    <row r="93" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="93" spans="1:11">
       <c r="A93" s="6">
         <v>92</v>
       </c>
@@ -5401,7 +5441,7 @@
       </c>
       <c r="K93" s="6"/>
     </row>
-    <row r="94" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="94" spans="1:11">
       <c r="A94" s="6">
         <v>93</v>
       </c>
@@ -5430,7 +5470,7 @@
       <c r="J94" s="6"/>
       <c r="K94" s="6"/>
     </row>
-    <row r="95" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="95" spans="1:11">
       <c r="A95" s="6">
         <v>94</v>
       </c>
@@ -5461,7 +5501,7 @@
       </c>
       <c r="K95" s="6"/>
     </row>
-    <row r="96" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="96" spans="1:11">
       <c r="A96" s="6">
         <v>95</v>
       </c>
@@ -5492,7 +5532,7 @@
       </c>
       <c r="K96" s="6"/>
     </row>
-    <row r="97" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="97" spans="1:11">
       <c r="A97" s="6">
         <v>96</v>
       </c>
@@ -5523,7 +5563,7 @@
       </c>
       <c r="K97" s="6"/>
     </row>
-    <row r="98" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="98" spans="1:11">
       <c r="A98" s="6">
         <v>97</v>
       </c>
@@ -5554,7 +5594,7 @@
       </c>
       <c r="K98" s="6"/>
     </row>
-    <row r="99" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="99" spans="1:11">
       <c r="A99" s="6">
         <v>98</v>
       </c>
@@ -5585,7 +5625,7 @@
       </c>
       <c r="K99" s="6"/>
     </row>
-    <row r="100" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="100" spans="1:11">
       <c r="A100" s="6">
         <v>99</v>
       </c>
@@ -5614,7 +5654,7 @@
       </c>
       <c r="K100" s="6"/>
     </row>
-    <row r="101" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="101" spans="1:11">
       <c r="A101" s="6">
         <v>100</v>
       </c>
@@ -5643,7 +5683,7 @@
       </c>
       <c r="K101" s="6"/>
     </row>
-    <row r="102" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="102" spans="1:11">
       <c r="A102" s="6">
         <v>101</v>
       </c>
@@ -5672,7 +5712,7 @@
       </c>
       <c r="K102" s="6"/>
     </row>
-    <row r="103" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="103" spans="1:11">
       <c r="A103" s="6">
         <v>102</v>
       </c>
@@ -5701,7 +5741,7 @@
       </c>
       <c r="K103" s="6"/>
     </row>
-    <row r="104" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="104" spans="1:11">
       <c r="A104" s="6">
         <v>103</v>
       </c>
@@ -5730,7 +5770,7 @@
       </c>
       <c r="K104" s="6"/>
     </row>
-    <row r="105" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="105" spans="1:11">
       <c r="A105" s="6">
         <v>104</v>
       </c>
@@ -5759,7 +5799,7 @@
       </c>
       <c r="K105" s="6"/>
     </row>
-    <row r="106" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="106" spans="1:11">
       <c r="A106" s="6">
         <v>105</v>
       </c>
@@ -5788,7 +5828,7 @@
       </c>
       <c r="K106" s="6"/>
     </row>
-    <row r="107" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="107" spans="1:11">
       <c r="A107" s="6">
         <v>106</v>
       </c>
@@ -5817,7 +5857,7 @@
       </c>
       <c r="K107" s="6"/>
     </row>
-    <row r="108" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="108" spans="1:11">
       <c r="A108" s="6">
         <v>107</v>
       </c>
@@ -5850,7 +5890,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="109" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="109" spans="1:11">
       <c r="A109" s="6">
         <v>108</v>
       </c>
@@ -5879,7 +5919,7 @@
       </c>
       <c r="K109" s="6"/>
     </row>
-    <row r="110" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="110" spans="1:11">
       <c r="A110" s="6">
         <v>109</v>
       </c>
@@ -5912,7 +5952,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="111" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="111" spans="1:11">
       <c r="A111" s="6">
         <v>110</v>
       </c>
@@ -5945,7 +5985,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="112" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="112" spans="1:11">
       <c r="A112" s="6">
         <v>111</v>
       </c>
@@ -5978,7 +6018,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="113" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="113" spans="1:12">
       <c r="A113" s="6">
         <v>112</v>
       </c>
@@ -6011,7 +6051,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="114" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="114" spans="1:12">
       <c r="A114" s="6">
         <v>113</v>
       </c>
@@ -6038,7 +6078,7 @@
       <c r="J114" s="6"/>
       <c r="K114" s="6"/>
     </row>
-    <row r="115" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="115" spans="1:12">
       <c r="A115" s="6">
         <v>114</v>
       </c>
@@ -6065,7 +6105,7 @@
       <c r="J115" s="6"/>
       <c r="K115" s="6"/>
     </row>
-    <row r="116" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="116" spans="1:12">
       <c r="A116" s="6">
         <v>115</v>
       </c>
@@ -6092,7 +6132,7 @@
       <c r="J116" s="6"/>
       <c r="K116" s="6"/>
     </row>
-    <row r="117" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="117" spans="1:12">
       <c r="A117" s="6">
         <v>116</v>
       </c>
@@ -6126,7 +6166,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="118" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="118" spans="1:12">
       <c r="A118" s="6">
         <v>117</v>
       </c>
@@ -6159,7 +6199,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="119" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="119" spans="1:12">
       <c r="A119" s="6">
         <v>118</v>
       </c>
@@ -6201,8 +6241,8 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:H82"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:H92"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
     <col min="2" max="2" width="34" customWidth="1"/>
@@ -6213,7 +6253,7 @@
     <col min="7" max="7" width="40" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="26" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:8" ht="26" customHeight="1">
       <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
@@ -6239,7 +6279,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="28" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:8" ht="28" customHeight="1">
       <c r="A2" s="10">
         <v>1</v>
       </c>
@@ -6262,7 +6302,7 @@
         <v>379</v>
       </c>
     </row>
-    <row r="3" spans="1:8" ht="42" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:8" ht="42" customHeight="1">
       <c r="A3" s="9">
         <v>2</v>
       </c>
@@ -6285,7 +6325,7 @@
         <v>381</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="70" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:8" ht="70" customHeight="1">
       <c r="A4" s="9">
         <v>3</v>
       </c>
@@ -6308,7 +6348,7 @@
         <v>384</v>
       </c>
     </row>
-    <row r="5" spans="1:8" ht="70" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:8" ht="70" customHeight="1">
       <c r="A5" s="9">
         <v>4</v>
       </c>
@@ -6331,7 +6371,7 @@
         <v>386</v>
       </c>
     </row>
-    <row r="6" spans="1:8" ht="28" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:8" ht="28" customHeight="1">
       <c r="A6" s="9">
         <v>5</v>
       </c>
@@ -6354,7 +6394,7 @@
         <v>388</v>
       </c>
     </row>
-    <row r="7" spans="1:8" ht="28" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:8" ht="28" customHeight="1">
       <c r="A7" s="9">
         <v>6</v>
       </c>
@@ -6377,7 +6417,7 @@
         <v>388</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:8">
       <c r="A8" s="9">
         <v>7</v>
       </c>
@@ -6398,7 +6438,7 @@
       </c>
       <c r="G8" s="8"/>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:8">
       <c r="A9" s="9">
         <v>8</v>
       </c>
@@ -6419,81 +6459,75 @@
       </c>
       <c r="G9" s="8"/>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:8">
       <c r="A10" s="9">
         <v>9</v>
       </c>
-      <c r="B10" s="8" t="s">
+      <c r="B10" s="22" t="s">
+        <v>496</v>
+      </c>
+      <c r="C10" s="8" t="s">
         <v>393</v>
       </c>
-      <c r="C10" s="8" t="s">
+      <c r="D10" s="8" t="s">
         <v>394</v>
-      </c>
-      <c r="D10" s="8" t="s">
-        <v>395</v>
       </c>
       <c r="E10" s="8" t="s">
         <v>86</v>
       </c>
       <c r="F10" s="9"/>
-      <c r="G10" s="8" t="s">
-        <v>406</v>
-      </c>
-    </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="G10" s="8"/>
+    </row>
+    <row r="11" spans="1:8">
       <c r="A11" s="9">
         <v>10</v>
       </c>
-      <c r="B11" s="8" t="s">
-        <v>396</v>
+      <c r="B11" s="22" t="s">
+        <v>497</v>
       </c>
       <c r="C11" s="8" t="s">
+        <v>393</v>
+      </c>
+      <c r="D11" s="8" t="s">
         <v>394</v>
-      </c>
-      <c r="D11" s="8" t="s">
-        <v>395</v>
       </c>
       <c r="E11" s="8" t="s">
         <v>86</v>
       </c>
       <c r="F11" s="9"/>
-      <c r="G11" s="8" t="s">
-        <v>406</v>
-      </c>
-    </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="G11" s="8"/>
+    </row>
+    <row r="12" spans="1:8">
       <c r="A12" s="9">
         <v>11</v>
       </c>
-      <c r="B12" s="8" t="s">
-        <v>397</v>
+      <c r="B12" s="22" t="s">
+        <v>498</v>
       </c>
       <c r="C12" s="8" t="s">
+        <v>393</v>
+      </c>
+      <c r="D12" s="8" t="s">
         <v>394</v>
-      </c>
-      <c r="D12" s="8" t="s">
-        <v>395</v>
       </c>
       <c r="E12" s="8" t="s">
         <v>86</v>
       </c>
       <c r="F12" s="9"/>
-      <c r="G12" s="8" t="s">
-        <v>406</v>
-      </c>
-    </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="G12" s="8"/>
+    </row>
+    <row r="13" spans="1:8">
       <c r="A13" s="9">
         <v>12</v>
       </c>
       <c r="B13" s="8" t="s">
-        <v>398</v>
+        <v>395</v>
       </c>
       <c r="C13" s="8" t="s">
         <v>69</v>
       </c>
       <c r="D13" s="8" t="s">
-        <v>399</v>
+        <v>396</v>
       </c>
       <c r="E13" s="8" t="s">
         <v>86</v>
@@ -6503,18 +6537,18 @@
       </c>
       <c r="G13" s="8"/>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:8">
       <c r="A14" s="9">
         <v>13</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>400</v>
+        <v>397</v>
       </c>
       <c r="C14" s="8" t="s">
         <v>69</v>
       </c>
       <c r="D14" s="8" t="s">
-        <v>399</v>
+        <v>396</v>
       </c>
       <c r="E14" s="8" t="s">
         <v>86</v>
@@ -6524,12 +6558,12 @@
       </c>
       <c r="G14" s="8"/>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:8">
       <c r="A15" s="9">
         <v>14</v>
       </c>
       <c r="B15" s="8" t="s">
-        <v>401</v>
+        <v>398</v>
       </c>
       <c r="C15" s="8" t="s">
         <v>69</v>
@@ -6545,18 +6579,18 @@
       </c>
       <c r="G15" s="8"/>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:8">
       <c r="A16" s="9">
         <v>15</v>
       </c>
       <c r="B16" s="8" t="s">
-        <v>402</v>
+        <v>399</v>
       </c>
       <c r="C16" s="8" t="s">
         <v>69</v>
       </c>
       <c r="D16" s="8" t="s">
-        <v>399</v>
+        <v>396</v>
       </c>
       <c r="E16" s="8" t="s">
         <v>86</v>
@@ -6566,18 +6600,18 @@
       </c>
       <c r="G16" s="8"/>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:7">
       <c r="A17" s="9">
         <v>16</v>
       </c>
       <c r="B17" s="8" t="s">
-        <v>403</v>
+        <v>400</v>
       </c>
       <c r="C17" s="8" t="s">
         <v>69</v>
       </c>
       <c r="D17" s="8" t="s">
-        <v>399</v>
+        <v>396</v>
       </c>
       <c r="E17" s="8" t="s">
         <v>86</v>
@@ -6587,18 +6621,18 @@
       </c>
       <c r="G17" s="8"/>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:7">
       <c r="A18" s="9">
         <v>17</v>
       </c>
       <c r="B18" s="8" t="s">
-        <v>404</v>
+        <v>401</v>
       </c>
       <c r="C18" s="8" t="s">
         <v>238</v>
       </c>
       <c r="D18" s="8" t="s">
-        <v>405</v>
+        <v>402</v>
       </c>
       <c r="E18" s="8" t="s">
         <v>68</v>
@@ -6608,12 +6642,12 @@
       </c>
       <c r="G18" s="8"/>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:7">
       <c r="A19" s="9">
         <v>18</v>
       </c>
-      <c r="B19" s="8" t="s">
-        <v>442</v>
+      <c r="B19" t="s">
+        <v>502</v>
       </c>
       <c r="C19" s="8" t="s">
         <v>38</v>
@@ -6626,15 +6660,15 @@
       </c>
       <c r="F19" s="9"/>
       <c r="G19" s="8" t="s">
-        <v>406</v>
-      </c>
-    </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.2">
+        <v>403</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7">
       <c r="A20" s="9">
         <v>19</v>
       </c>
-      <c r="B20" s="8" t="s">
-        <v>443</v>
+      <c r="B20" t="s">
+        <v>503</v>
       </c>
       <c r="C20" s="8" t="s">
         <v>38</v>
@@ -6647,15 +6681,15 @@
       </c>
       <c r="F20" s="9"/>
       <c r="G20" s="8" t="s">
-        <v>406</v>
-      </c>
-    </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.2">
+        <v>403</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7">
       <c r="A21" s="9">
         <v>20</v>
       </c>
-      <c r="B21" s="8" t="s">
-        <v>444</v>
+      <c r="B21" t="s">
+        <v>504</v>
       </c>
       <c r="C21" s="8" t="s">
         <v>38</v>
@@ -6668,21 +6702,21 @@
       </c>
       <c r="F21" s="9"/>
       <c r="G21" s="8" t="s">
-        <v>406</v>
-      </c>
-    </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.2">
+        <v>403</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7">
       <c r="A22" s="9">
         <v>21</v>
       </c>
       <c r="B22" s="8" t="s">
-        <v>419</v>
+        <v>416</v>
       </c>
       <c r="C22" s="8" t="s">
         <v>238</v>
       </c>
       <c r="D22" s="8" t="s">
-        <v>405</v>
+        <v>402</v>
       </c>
       <c r="E22" s="8" t="s">
         <v>68</v>
@@ -6692,18 +6726,18 @@
       </c>
       <c r="G22" s="8"/>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:7">
       <c r="A23" s="9">
         <v>22</v>
       </c>
       <c r="B23" s="8" t="s">
-        <v>420</v>
+        <v>417</v>
       </c>
       <c r="C23" s="8" t="s">
         <v>238</v>
       </c>
       <c r="D23" s="8" t="s">
-        <v>405</v>
+        <v>402</v>
       </c>
       <c r="E23" s="8" t="s">
         <v>68</v>
@@ -6713,12 +6747,12 @@
       </c>
       <c r="G23" s="8"/>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:7">
       <c r="A24" s="9">
         <v>23</v>
       </c>
       <c r="B24" s="8" t="s">
-        <v>421</v>
+        <v>418</v>
       </c>
       <c r="C24" s="7" t="s">
         <v>159</v>
@@ -6734,12 +6768,12 @@
       </c>
       <c r="G24" s="8"/>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:7">
       <c r="A25" s="9">
         <v>24</v>
       </c>
       <c r="B25" s="8" t="s">
-        <v>429</v>
+        <v>426</v>
       </c>
       <c r="C25" s="8" t="s">
         <v>242</v>
@@ -6755,12 +6789,12 @@
       </c>
       <c r="G25" s="8"/>
     </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:7">
       <c r="A26" s="9">
         <v>25</v>
       </c>
       <c r="B26" s="8" t="s">
-        <v>422</v>
+        <v>419</v>
       </c>
       <c r="C26" s="7" t="s">
         <v>177</v>
@@ -6776,12 +6810,12 @@
       </c>
       <c r="G26" s="8"/>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:7">
       <c r="A27" s="9">
         <v>26</v>
       </c>
       <c r="B27" s="8" t="s">
-        <v>430</v>
+        <v>427</v>
       </c>
       <c r="C27" s="7" t="s">
         <v>186</v>
@@ -6797,12 +6831,12 @@
       </c>
       <c r="G27" s="8"/>
     </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:7">
       <c r="A28" s="9">
         <v>27</v>
       </c>
       <c r="B28" s="8" t="s">
-        <v>431</v>
+        <v>428</v>
       </c>
       <c r="C28" s="7" t="s">
         <v>186</v>
@@ -6818,12 +6852,12 @@
       </c>
       <c r="G28" s="8"/>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:7">
       <c r="A29" s="9">
         <v>28</v>
       </c>
       <c r="B29" s="8" t="s">
-        <v>432</v>
+        <v>429</v>
       </c>
       <c r="C29" s="8" t="s">
         <v>242</v>
@@ -6839,12 +6873,12 @@
       </c>
       <c r="G29" s="8"/>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:7">
       <c r="A30" s="9">
         <v>29</v>
       </c>
       <c r="B30" s="8" t="s">
-        <v>433</v>
+        <v>430</v>
       </c>
       <c r="C30" s="7" t="s">
         <v>231</v>
@@ -6860,12 +6894,12 @@
       </c>
       <c r="G30" s="8"/>
     </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:7">
       <c r="A31" s="9">
         <v>30</v>
       </c>
       <c r="B31" s="8" t="s">
-        <v>434</v>
+        <v>431</v>
       </c>
       <c r="C31" s="7" t="s">
         <v>231</v>
@@ -6881,12 +6915,12 @@
       </c>
       <c r="G31" s="8"/>
     </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:7">
       <c r="A32" s="9">
         <v>31</v>
       </c>
       <c r="B32" s="8" t="s">
-        <v>435</v>
+        <v>432</v>
       </c>
       <c r="C32" s="7" t="s">
         <v>231</v>
@@ -6902,12 +6936,12 @@
       </c>
       <c r="G32" s="8"/>
     </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:7">
       <c r="A33" s="9">
         <v>32</v>
       </c>
       <c r="B33" s="8" t="s">
-        <v>436</v>
+        <v>433</v>
       </c>
       <c r="C33" s="7" t="s">
         <v>231</v>
@@ -6923,12 +6957,12 @@
       </c>
       <c r="G33" s="8"/>
     </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:7">
       <c r="A34" s="9">
         <v>33</v>
       </c>
       <c r="B34" s="8" t="s">
-        <v>437</v>
+        <v>434</v>
       </c>
       <c r="C34" s="7" t="s">
         <v>231</v>
@@ -6944,12 +6978,12 @@
       </c>
       <c r="G34" s="8"/>
     </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:7">
       <c r="A35" s="9">
         <v>34</v>
       </c>
       <c r="B35" s="8" t="s">
-        <v>438</v>
+        <v>435</v>
       </c>
       <c r="C35" s="7" t="s">
         <v>231</v>
@@ -6965,12 +6999,12 @@
       </c>
       <c r="G35" s="8"/>
     </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:7">
       <c r="A36" s="9">
         <v>35</v>
       </c>
       <c r="B36" s="8" t="s">
-        <v>439</v>
+        <v>436</v>
       </c>
       <c r="C36" s="7" t="s">
         <v>231</v>
@@ -6986,12 +7020,12 @@
       </c>
       <c r="G36" s="8"/>
     </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:7">
       <c r="A37" s="9">
         <v>36</v>
       </c>
       <c r="B37" s="8" t="s">
-        <v>440</v>
+        <v>437</v>
       </c>
       <c r="C37" s="7" t="s">
         <v>231</v>
@@ -7007,12 +7041,12 @@
       </c>
       <c r="G37" s="8"/>
     </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:7">
       <c r="A38" s="9">
         <v>37</v>
       </c>
       <c r="B38" s="8" t="s">
-        <v>469</v>
+        <v>463</v>
       </c>
       <c r="C38" s="8" t="s">
         <v>69</v>
@@ -7025,15 +7059,15 @@
       </c>
       <c r="F38" s="9"/>
       <c r="G38" s="8" t="s">
-        <v>406</v>
-      </c>
-    </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.2">
+        <v>403</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7">
       <c r="A39" s="9">
         <v>38</v>
       </c>
       <c r="B39" s="8" t="s">
-        <v>470</v>
+        <v>464</v>
       </c>
       <c r="C39" s="8" t="s">
         <v>69</v>
@@ -7046,15 +7080,15 @@
       </c>
       <c r="F39" s="9"/>
       <c r="G39" s="8" t="s">
-        <v>406</v>
-      </c>
-    </row>
-    <row r="40" spans="1:7" x14ac:dyDescent="0.2">
+        <v>403</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7">
       <c r="A40" s="9">
         <v>39</v>
       </c>
       <c r="B40" s="8" t="s">
-        <v>446</v>
+        <v>440</v>
       </c>
       <c r="C40" s="8" t="s">
         <v>238</v>
@@ -7070,12 +7104,12 @@
       </c>
       <c r="G40" s="8"/>
     </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:7">
       <c r="A41" s="9">
         <v>40</v>
       </c>
       <c r="B41" s="8" t="s">
-        <v>447</v>
+        <v>441</v>
       </c>
       <c r="C41" s="8" t="s">
         <v>238</v>
@@ -7091,18 +7125,18 @@
       </c>
       <c r="G41" s="8"/>
     </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:7">
       <c r="A42" s="9">
         <v>41</v>
       </c>
       <c r="B42" s="8" t="s">
-        <v>445</v>
+        <v>439</v>
       </c>
       <c r="C42" s="8" t="s">
         <v>238</v>
       </c>
       <c r="D42" s="8" t="s">
-        <v>405</v>
+        <v>402</v>
       </c>
       <c r="E42" s="8" t="s">
         <v>86</v>
@@ -7112,15 +7146,15 @@
       </c>
       <c r="G42" s="8"/>
     </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:7">
       <c r="A43" s="9">
         <v>42</v>
       </c>
       <c r="B43" s="14" t="s">
-        <v>475</v>
+        <v>469</v>
       </c>
       <c r="C43" s="14" t="s">
-        <v>448</v>
+        <v>442</v>
       </c>
       <c r="D43" s="14" t="s">
         <v>269</v>
@@ -7129,18 +7163,18 @@
         <v>86</v>
       </c>
       <c r="G43" s="8" t="s">
-        <v>406</v>
-      </c>
-    </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.2">
+        <v>403</v>
+      </c>
+    </row>
+    <row r="44" spans="1:7">
       <c r="A44" s="9">
         <v>43</v>
       </c>
       <c r="B44" s="14" t="s">
-        <v>477</v>
+        <v>471</v>
       </c>
       <c r="C44" s="14" t="s">
-        <v>449</v>
+        <v>443</v>
       </c>
       <c r="D44" s="14" t="s">
         <v>242</v>
@@ -7149,18 +7183,18 @@
         <v>86</v>
       </c>
       <c r="G44" s="8" t="s">
-        <v>406</v>
-      </c>
-    </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.2">
+        <v>403</v>
+      </c>
+    </row>
+    <row r="45" spans="1:7">
       <c r="A45" s="9">
         <v>44</v>
       </c>
       <c r="B45" s="14" t="s">
-        <v>455</v>
+        <v>449</v>
       </c>
       <c r="C45" s="14" t="s">
-        <v>450</v>
+        <v>444</v>
       </c>
       <c r="D45" s="14" t="s">
         <v>64</v>
@@ -7172,12 +7206,12 @@
         <v>1</v>
       </c>
     </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:7">
       <c r="A46" s="9">
         <v>45</v>
       </c>
       <c r="B46" t="s">
-        <v>451</v>
+        <v>445</v>
       </c>
       <c r="C46" s="7" t="s">
         <v>186</v>
@@ -7192,15 +7226,15 @@
         <v>2</v>
       </c>
     </row>
-    <row r="47" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:7">
       <c r="A47" s="9">
         <v>46</v>
       </c>
       <c r="B47" s="14" t="s">
-        <v>452</v>
+        <v>446</v>
       </c>
       <c r="C47" s="14" t="s">
-        <v>449</v>
+        <v>443</v>
       </c>
       <c r="D47" t="s">
         <v>283</v>
@@ -7209,18 +7243,18 @@
         <v>86</v>
       </c>
       <c r="G47" s="8" t="s">
-        <v>406</v>
-      </c>
-    </row>
-    <row r="48" spans="1:7" x14ac:dyDescent="0.2">
+        <v>403</v>
+      </c>
+    </row>
+    <row r="48" spans="1:7">
       <c r="A48" s="9">
         <v>47</v>
       </c>
       <c r="B48" s="14" t="s">
-        <v>453</v>
+        <v>447</v>
       </c>
       <c r="C48" s="14" t="s">
-        <v>458</v>
+        <v>452</v>
       </c>
       <c r="D48" t="s">
         <v>269</v>
@@ -7232,15 +7266,15 @@
         <v>2</v>
       </c>
     </row>
-    <row r="49" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:7">
       <c r="A49" s="9">
         <v>48</v>
       </c>
       <c r="B49" s="14" t="s">
-        <v>454</v>
+        <v>448</v>
       </c>
       <c r="C49" s="14" t="s">
-        <v>458</v>
+        <v>452</v>
       </c>
       <c r="D49" t="s">
         <v>269</v>
@@ -7252,15 +7286,15 @@
         <v>2</v>
       </c>
     </row>
-    <row r="50" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:7">
       <c r="A50" s="9">
         <v>49</v>
       </c>
       <c r="B50" s="14" t="s">
-        <v>456</v>
+        <v>450</v>
       </c>
       <c r="C50" s="14" t="s">
-        <v>450</v>
+        <v>444</v>
       </c>
       <c r="D50" t="s">
         <v>269</v>
@@ -7272,15 +7306,15 @@
         <v>1</v>
       </c>
     </row>
-    <row r="51" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:7">
       <c r="A51" s="9">
         <v>50</v>
       </c>
       <c r="B51" s="14" t="s">
-        <v>459</v>
+        <v>453</v>
       </c>
       <c r="C51" s="14" t="s">
-        <v>448</v>
+        <v>442</v>
       </c>
       <c r="D51" s="14" t="s">
         <v>64</v>
@@ -7292,15 +7326,15 @@
         <v>1</v>
       </c>
     </row>
-    <row r="52" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:7">
       <c r="A52" s="9">
         <v>51</v>
       </c>
       <c r="B52" s="14" t="s">
-        <v>457</v>
+        <v>451</v>
       </c>
       <c r="C52" s="14" t="s">
-        <v>450</v>
+        <v>444</v>
       </c>
       <c r="D52" t="s">
         <v>269</v>
@@ -7312,15 +7346,15 @@
         <v>1</v>
       </c>
     </row>
-    <row r="53" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:7">
       <c r="A53" s="16">
         <v>52</v>
       </c>
       <c r="B53" s="14" t="s">
-        <v>460</v>
+        <v>454</v>
       </c>
       <c r="C53" s="14" t="s">
-        <v>448</v>
+        <v>442</v>
       </c>
       <c r="D53" t="s">
         <v>269</v>
@@ -7332,18 +7366,18 @@
         <v>1</v>
       </c>
     </row>
-    <row r="54" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:7">
       <c r="A54" s="16">
         <v>53</v>
       </c>
       <c r="B54" s="14" t="s">
-        <v>492</v>
+        <v>486</v>
       </c>
       <c r="C54" s="14" t="s">
-        <v>491</v>
+        <v>485</v>
       </c>
       <c r="D54" s="14" t="s">
-        <v>493</v>
+        <v>487</v>
       </c>
       <c r="E54" s="8" t="s">
         <v>86</v>
@@ -7352,18 +7386,18 @@
         <v>1</v>
       </c>
     </row>
-    <row r="55" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:7">
       <c r="A55" s="16">
         <v>54</v>
       </c>
       <c r="B55" s="14" t="s">
-        <v>461</v>
+        <v>455</v>
       </c>
       <c r="C55" s="14" t="s">
-        <v>463</v>
+        <v>457</v>
       </c>
       <c r="D55" t="s">
-        <v>462</v>
+        <v>456</v>
       </c>
       <c r="E55" s="8" t="s">
         <v>86</v>
@@ -7372,36 +7406,36 @@
         <v>20</v>
       </c>
     </row>
-    <row r="56" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:7">
       <c r="A56" s="18">
         <v>55</v>
       </c>
       <c r="B56" s="14" t="s">
-        <v>464</v>
+        <v>458</v>
       </c>
       <c r="C56" s="14" t="s">
-        <v>450</v>
+        <v>444</v>
       </c>
       <c r="D56" t="s">
-        <v>465</v>
+        <v>459</v>
       </c>
       <c r="E56" s="8" t="s">
         <v>86</v>
       </c>
       <c r="F56" s="20"/>
       <c r="G56" s="8" t="s">
-        <v>406</v>
-      </c>
-    </row>
-    <row r="57" spans="1:7" x14ac:dyDescent="0.2">
+        <v>403</v>
+      </c>
+    </row>
+    <row r="57" spans="1:7">
       <c r="A57" s="19">
         <v>56</v>
       </c>
       <c r="B57" s="14" t="s">
-        <v>466</v>
+        <v>460</v>
       </c>
       <c r="C57" s="14" t="s">
-        <v>450</v>
+        <v>444</v>
       </c>
       <c r="D57" t="s">
         <v>269</v>
@@ -7413,15 +7447,15 @@
         <v>1</v>
       </c>
     </row>
-    <row r="58" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:7">
       <c r="A58" s="19">
         <v>56</v>
       </c>
       <c r="B58" s="22" t="s">
-        <v>467</v>
+        <v>461</v>
       </c>
       <c r="C58" s="14" t="s">
-        <v>472</v>
+        <v>466</v>
       </c>
       <c r="D58" t="s">
         <v>269</v>
@@ -7433,15 +7467,15 @@
         <v>2</v>
       </c>
     </row>
-    <row r="59" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:7">
       <c r="A59" s="19">
         <v>56</v>
       </c>
       <c r="B59" s="22" t="s">
-        <v>468</v>
+        <v>462</v>
       </c>
       <c r="C59" s="14" t="s">
-        <v>472</v>
+        <v>466</v>
       </c>
       <c r="D59" t="s">
         <v>269</v>
@@ -7453,15 +7487,15 @@
         <v>2</v>
       </c>
     </row>
-    <row r="60" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:7">
       <c r="A60" s="19">
         <v>57</v>
       </c>
       <c r="B60" s="14" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="C60" s="14" t="s">
-        <v>472</v>
+        <v>466</v>
       </c>
       <c r="D60" t="s">
         <v>269</v>
@@ -7473,15 +7507,15 @@
         <v>1</v>
       </c>
     </row>
-    <row r="61" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:7">
       <c r="A61" s="19">
         <v>58</v>
       </c>
       <c r="B61" s="14" t="s">
-        <v>471</v>
+        <v>465</v>
       </c>
       <c r="C61" s="14" t="s">
-        <v>472</v>
+        <v>466</v>
       </c>
       <c r="D61" t="s">
         <v>269</v>
@@ -7493,15 +7527,15 @@
         <v>1</v>
       </c>
     </row>
-    <row r="62" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:7">
       <c r="A62" s="19">
         <v>59</v>
       </c>
       <c r="B62" s="14" t="s">
-        <v>473</v>
+        <v>467</v>
       </c>
       <c r="C62" s="14" t="s">
-        <v>449</v>
+        <v>443</v>
       </c>
       <c r="D62" t="s">
         <v>269</v>
@@ -7513,15 +7547,15 @@
         <v>1</v>
       </c>
     </row>
-    <row r="63" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:7">
       <c r="A63" s="19">
         <v>60</v>
       </c>
       <c r="B63" s="14" t="s">
-        <v>474</v>
+        <v>468</v>
       </c>
       <c r="C63" s="14" t="s">
-        <v>448</v>
+        <v>442</v>
       </c>
       <c r="D63" t="s">
         <v>149</v>
@@ -7530,18 +7564,18 @@
         <v>86</v>
       </c>
       <c r="G63" s="8" t="s">
-        <v>406</v>
-      </c>
-    </row>
-    <row r="64" spans="1:7" x14ac:dyDescent="0.2">
+        <v>403</v>
+      </c>
+    </row>
+    <row r="64" spans="1:7">
       <c r="A64" s="19">
         <v>61</v>
       </c>
       <c r="B64" s="14" t="s">
-        <v>476</v>
+        <v>470</v>
       </c>
       <c r="C64" s="14" t="s">
-        <v>458</v>
+        <v>452</v>
       </c>
       <c r="D64" t="s">
         <v>269</v>
@@ -7549,20 +7583,20 @@
       <c r="E64" s="8" t="s">
         <v>86</v>
       </c>
-      <c r="F64" s="24">
+      <c r="F64" s="18">
         <v>1</v>
       </c>
       <c r="G64" s="8"/>
     </row>
-    <row r="65" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:7">
       <c r="A65" s="19">
         <v>62</v>
       </c>
       <c r="B65" s="14" t="s">
-        <v>478</v>
+        <v>472</v>
       </c>
       <c r="C65" s="14" t="s">
-        <v>448</v>
+        <v>442</v>
       </c>
       <c r="D65" t="s">
         <v>269</v>
@@ -7571,18 +7605,18 @@
         <v>86</v>
       </c>
       <c r="G65" s="8" t="s">
-        <v>406</v>
-      </c>
-    </row>
-    <row r="66" spans="1:7" x14ac:dyDescent="0.2">
+        <v>403</v>
+      </c>
+    </row>
+    <row r="66" spans="1:7">
       <c r="A66" s="19">
         <v>63</v>
       </c>
       <c r="B66" s="14" t="s">
-        <v>479</v>
+        <v>473</v>
       </c>
       <c r="C66" s="14" t="s">
-        <v>449</v>
+        <v>443</v>
       </c>
       <c r="D66" t="s">
         <v>64</v>
@@ -7595,15 +7629,15 @@
       </c>
       <c r="G66" s="8"/>
     </row>
-    <row r="67" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:7">
       <c r="A67" s="19">
         <v>64</v>
       </c>
       <c r="B67" s="14" t="s">
-        <v>480</v>
+        <v>474</v>
       </c>
       <c r="C67" s="23" t="s">
-        <v>458</v>
+        <v>452</v>
       </c>
       <c r="D67" t="s">
         <v>269</v>
@@ -7616,35 +7650,35 @@
       </c>
       <c r="G67" s="8"/>
     </row>
-    <row r="68" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="68" spans="1:7">
       <c r="A68" s="19">
         <v>65</v>
       </c>
       <c r="B68" s="14" t="s">
-        <v>481</v>
+        <v>475</v>
       </c>
       <c r="C68" s="23" t="s">
-        <v>448</v>
+        <v>442</v>
       </c>
       <c r="D68" t="s">
-        <v>497</v>
+        <v>491</v>
       </c>
       <c r="E68" s="8" t="s">
         <v>86</v>
       </c>
       <c r="G68" s="8" t="s">
-        <v>406</v>
-      </c>
-    </row>
-    <row r="69" spans="1:7" x14ac:dyDescent="0.2">
+        <v>403</v>
+      </c>
+    </row>
+    <row r="69" spans="1:7">
       <c r="A69" s="19">
         <v>66</v>
       </c>
       <c r="B69" s="14" t="s">
-        <v>482</v>
+        <v>476</v>
       </c>
       <c r="C69" s="23" t="s">
-        <v>458</v>
+        <v>452</v>
       </c>
       <c r="D69" t="s">
         <v>64</v>
@@ -7657,15 +7691,15 @@
       </c>
       <c r="G69" s="8"/>
     </row>
-    <row r="70" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="70" spans="1:7">
       <c r="A70" s="19">
         <v>67</v>
       </c>
       <c r="B70" s="14" t="s">
-        <v>483</v>
+        <v>477</v>
       </c>
       <c r="C70" s="23" t="s">
-        <v>449</v>
+        <v>443</v>
       </c>
       <c r="D70" t="s">
         <v>269</v>
@@ -7674,18 +7708,18 @@
         <v>86</v>
       </c>
       <c r="G70" s="8" t="s">
-        <v>406</v>
-      </c>
-    </row>
-    <row r="71" spans="1:7" x14ac:dyDescent="0.2">
+        <v>403</v>
+      </c>
+    </row>
+    <row r="71" spans="1:7">
       <c r="A71" s="19">
         <v>68</v>
       </c>
       <c r="B71" s="14" t="s">
-        <v>484</v>
+        <v>478</v>
       </c>
       <c r="C71" s="23" t="s">
-        <v>449</v>
+        <v>443</v>
       </c>
       <c r="D71" t="s">
         <v>269</v>
@@ -7694,18 +7728,18 @@
         <v>86</v>
       </c>
       <c r="G71" s="8" t="s">
-        <v>406</v>
-      </c>
-    </row>
-    <row r="72" spans="1:7" x14ac:dyDescent="0.2">
+        <v>403</v>
+      </c>
+    </row>
+    <row r="72" spans="1:7">
       <c r="A72" s="19">
         <v>69</v>
       </c>
       <c r="B72" s="14" t="s">
-        <v>485</v>
+        <v>479</v>
       </c>
       <c r="C72" s="23" t="s">
-        <v>486</v>
+        <v>480</v>
       </c>
       <c r="D72" t="s">
         <v>269</v>
@@ -7718,15 +7752,15 @@
       </c>
       <c r="G72" s="8"/>
     </row>
-    <row r="73" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="73" spans="1:7">
       <c r="A73" s="19">
         <v>70</v>
       </c>
       <c r="B73" s="14" t="s">
-        <v>487</v>
+        <v>481</v>
       </c>
       <c r="C73" s="23" t="s">
-        <v>486</v>
+        <v>480</v>
       </c>
       <c r="D73" t="s">
         <v>269</v>
@@ -7739,15 +7773,15 @@
       </c>
       <c r="G73" s="8"/>
     </row>
-    <row r="74" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="74" spans="1:7">
       <c r="A74" s="19">
         <v>71</v>
       </c>
       <c r="B74" s="14" t="s">
-        <v>496</v>
+        <v>490</v>
       </c>
       <c r="C74" s="23" t="s">
-        <v>486</v>
+        <v>480</v>
       </c>
       <c r="D74" t="s">
         <v>269</v>
@@ -7760,18 +7794,18 @@
       </c>
       <c r="G74" s="8"/>
     </row>
-    <row r="75" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="75" spans="1:7">
       <c r="A75" s="19">
         <v>72</v>
       </c>
       <c r="B75" s="14" t="s">
-        <v>488</v>
+        <v>482</v>
       </c>
       <c r="C75" s="23" t="s">
-        <v>491</v>
+        <v>485</v>
       </c>
       <c r="D75" t="s">
-        <v>495</v>
+        <v>489</v>
       </c>
       <c r="E75" s="8" t="s">
         <v>86</v>
@@ -7781,18 +7815,18 @@
       </c>
       <c r="G75" s="8"/>
     </row>
-    <row r="76" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="76" spans="1:7">
       <c r="A76" s="19">
         <v>73</v>
       </c>
       <c r="B76" s="14" t="s">
+        <v>483</v>
+      </c>
+      <c r="C76" s="23" t="s">
+        <v>485</v>
+      </c>
+      <c r="D76" t="s">
         <v>489</v>
-      </c>
-      <c r="C76" s="23" t="s">
-        <v>491</v>
-      </c>
-      <c r="D76" t="s">
-        <v>495</v>
       </c>
       <c r="E76" s="8" t="s">
         <v>86</v>
@@ -7802,18 +7836,18 @@
       </c>
       <c r="G76" s="8"/>
     </row>
-    <row r="77" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="77" spans="1:7">
       <c r="A77" s="19">
         <v>74</v>
       </c>
       <c r="B77" s="14" t="s">
-        <v>490</v>
+        <v>484</v>
       </c>
       <c r="C77" s="23" t="s">
-        <v>491</v>
+        <v>485</v>
       </c>
       <c r="D77" t="s">
-        <v>495</v>
+        <v>489</v>
       </c>
       <c r="E77" s="8" t="s">
         <v>86</v>
@@ -7823,15 +7857,15 @@
       </c>
       <c r="G77" s="8"/>
     </row>
-    <row r="78" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="78" spans="1:7">
       <c r="A78" s="19">
         <v>75</v>
       </c>
       <c r="B78" s="14" t="s">
-        <v>494</v>
+        <v>488</v>
       </c>
       <c r="C78" s="14" t="s">
-        <v>491</v>
+        <v>485</v>
       </c>
       <c r="D78" t="s">
         <v>306</v>
@@ -7844,15 +7878,15 @@
       </c>
       <c r="G78" s="8"/>
     </row>
-    <row r="79" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="79" spans="1:7">
       <c r="A79" s="19">
         <v>76</v>
       </c>
       <c r="B79" s="14" t="s">
-        <v>498</v>
+        <v>492</v>
       </c>
       <c r="C79" s="14" t="s">
-        <v>491</v>
+        <v>485</v>
       </c>
       <c r="D79" t="s">
         <v>264</v>
@@ -7865,15 +7899,15 @@
       </c>
       <c r="G79" s="8"/>
     </row>
-    <row r="80" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="80" spans="1:7">
       <c r="A80" s="19">
         <v>77</v>
       </c>
       <c r="B80" s="14" t="s">
-        <v>499</v>
+        <v>493</v>
       </c>
       <c r="C80" s="14" t="s">
-        <v>491</v>
+        <v>485</v>
       </c>
       <c r="D80" t="s">
         <v>269</v>
@@ -7885,18 +7919,18 @@
         <v>1</v>
       </c>
       <c r="G80" s="8" t="s">
-        <v>406</v>
-      </c>
-    </row>
-    <row r="81" spans="1:6" x14ac:dyDescent="0.2">
+        <v>403</v>
+      </c>
+    </row>
+    <row r="81" spans="1:7">
       <c r="A81" s="19">
         <v>78</v>
       </c>
       <c r="B81" s="14" t="s">
-        <v>500</v>
+        <v>494</v>
       </c>
       <c r="C81" s="14" t="s">
-        <v>491</v>
+        <v>485</v>
       </c>
       <c r="D81" t="s">
         <v>67</v>
@@ -7908,15 +7942,15 @@
         <v>1</v>
       </c>
     </row>
-    <row r="82" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="82" spans="1:7">
       <c r="A82" s="19">
         <v>79</v>
       </c>
       <c r="B82" s="14" t="s">
-        <v>501</v>
+        <v>495</v>
       </c>
       <c r="C82" s="14" t="s">
-        <v>491</v>
+        <v>485</v>
       </c>
       <c r="D82" t="s">
         <v>264</v>
@@ -7926,12 +7960,152 @@
       </c>
       <c r="F82">
         <v>1</v>
+      </c>
+    </row>
+    <row r="83" spans="1:7">
+      <c r="A83" s="19">
+        <v>80</v>
+      </c>
+      <c r="B83" s="24" t="s">
+        <v>499</v>
+      </c>
+      <c r="C83" s="8" t="s">
+        <v>393</v>
+      </c>
+      <c r="D83" t="s">
+        <v>44</v>
+      </c>
+      <c r="E83" s="8" t="s">
+        <v>86</v>
+      </c>
+      <c r="G83" s="8" t="s">
+        <v>403</v>
+      </c>
+    </row>
+    <row r="84" spans="1:7">
+      <c r="A84" s="19">
+        <v>81</v>
+      </c>
+      <c r="B84" t="s">
+        <v>501</v>
+      </c>
+      <c r="C84" s="8" t="s">
+        <v>393</v>
+      </c>
+      <c r="D84" t="s">
+        <v>44</v>
+      </c>
+      <c r="E84" s="8" t="s">
+        <v>86</v>
+      </c>
+      <c r="G84" s="8" t="s">
+        <v>403</v>
+      </c>
+    </row>
+    <row r="85" spans="1:7">
+      <c r="A85" s="19">
+        <v>82</v>
+      </c>
+      <c r="B85" t="s">
+        <v>500</v>
+      </c>
+      <c r="C85" s="8" t="s">
+        <v>393</v>
+      </c>
+      <c r="D85" t="s">
+        <v>44</v>
+      </c>
+      <c r="E85" s="8" t="s">
+        <v>86</v>
+      </c>
+      <c r="G85" s="8" t="s">
+        <v>403</v>
+      </c>
+    </row>
+    <row r="86" spans="1:7">
+      <c r="A86" s="19">
+        <v>83</v>
+      </c>
+      <c r="B86" t="s">
+        <v>505</v>
+      </c>
+      <c r="C86" s="8" t="s">
+        <v>506</v>
+      </c>
+      <c r="D86" t="s">
+        <v>44</v>
+      </c>
+      <c r="E86" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="G86" s="8" t="s">
+        <v>403</v>
+      </c>
+    </row>
+    <row r="87" spans="1:7">
+      <c r="A87" s="19">
+        <v>84</v>
+      </c>
+      <c r="B87" t="s">
+        <v>507</v>
+      </c>
+      <c r="C87" s="8" t="s">
+        <v>509</v>
+      </c>
+      <c r="D87" t="s">
+        <v>44</v>
+      </c>
+      <c r="E87" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="G87" s="8" t="s">
+        <v>403</v>
+      </c>
+    </row>
+    <row r="88" spans="1:7">
+      <c r="A88" s="19">
+        <v>85</v>
+      </c>
+      <c r="B88" t="s">
+        <v>508</v>
+      </c>
+      <c r="C88" s="8" t="s">
+        <v>509</v>
+      </c>
+      <c r="D88" t="s">
+        <v>44</v>
+      </c>
+      <c r="E88" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="G88" s="8" t="s">
+        <v>403</v>
+      </c>
+    </row>
+    <row r="89" spans="1:7">
+      <c r="A89" s="19">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="90" spans="1:7">
+      <c r="A90" s="19">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="91" spans="1:7">
+      <c r="A91" s="19">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="92" spans="1:7">
+      <c r="A92" s="19">
+        <v>89</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="10" type="noConversion"/>
   <dataValidations count="1">
-    <dataValidation type="list" errorTitle="Invalid brand" error="Choose yc, staple, or shared from the list." sqref="E3:E82" xr:uid="{00000000-0002-0000-0200-000000000000}">
+    <dataValidation type="list" errorTitle="Invalid brand" error="Choose yc, staple, or shared from the list." sqref="E3:E88" xr:uid="{00000000-0002-0000-0200-000000000000}">
       <formula1>"yc,staple,shared"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
NCD: Plain Yogurt 1kg (it-009) กลับมาขาย — ตั้ง Par NCD = 4
แพรกลับคำสั่งจากก่อนหน้า (70b2c34 — ตอนนั้นบอกว่าไม่มีขาย) เป็นให้ขายที่ NCD
Par 4 — แก้ par_levels(NCD) ใน Supabase ตรงๆ (ไม่ต้อง deploy โค้ด มีผลทันที)
+ ไฟล์ Excel ให้ตรงกัน คืนสีตัวอักษรปกติ (จากสีจางที่เคยทำไว้ตอน "ไม่มีขาย")
จัดเรียงใหม่ย้ายกลับไปกลุ่ม "มีขาย" ในหมวด Yogurt 1kg/Box — แถบหัวหมวดกลับไป
นับ "มีที่ NCD 3" ถูกต้อง (จาก 2)
</commit_message>
<xml_diff>
--- a/NCD_Brand_Tagging.xlsx
+++ b/NCD_Brand_Tagging.xlsx
@@ -18,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="17">
+  <fonts count="18">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -118,6 +118,10 @@
       <name val="Arial"/>
       <b val="1"/>
       <color rgb="FF5A2E1B"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
       <sz val="11"/>
     </font>
   </fonts>
@@ -225,7 +229,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="44">
+  <cellXfs count="47">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -336,6 +340,13 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="15" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1193,7 +1204,7 @@
     <row r="2" ht="20" customHeight="1" s="28">
       <c r="A2" s="34" t="inlineStr">
         <is>
-          <t>Yogurt 1kg/Box  (9 รายการ · มีที่ NCD 2 · คอลัมน์ซ้าย)</t>
+          <t>Yogurt 1kg/Box  (9 รายการ · มีที่ NCD 3 · คอลัมน์ซ้าย)</t>
         </is>
       </c>
       <c r="B2" s="26" t="n"/>
@@ -1300,47 +1311,49 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="29" t="n">
+      <c r="A5" s="41" t="n">
         <v>3</v>
       </c>
-      <c r="B5" s="30" t="inlineStr">
+      <c r="B5" s="42" t="inlineStr">
         <is>
           <t>it-009</t>
         </is>
       </c>
-      <c r="C5" s="30" t="inlineStr">
+      <c r="C5" s="42" t="inlineStr">
         <is>
           <t>Yogurt 1kg/Box</t>
         </is>
       </c>
-      <c r="D5" s="30" t="inlineStr">
+      <c r="D5" s="42" t="inlineStr">
         <is>
           <t>Plain Yogurt (ธรรมชาติ)</t>
         </is>
       </c>
-      <c r="E5" s="31" t="n"/>
-      <c r="F5" s="30" t="inlineStr">
+      <c r="E5" s="44" t="n"/>
+      <c r="F5" s="42" t="inlineStr">
         <is>
           <t>1kg/Box</t>
         </is>
       </c>
-      <c r="G5" s="32" t="n"/>
-      <c r="H5" s="32" t="inlineStr">
-        <is>
-          <t>yc</t>
-        </is>
-      </c>
-      <c r="I5" s="29" t="n">
+      <c r="G5" s="45" t="n">
+        <v>4</v>
+      </c>
+      <c r="H5" s="45" t="inlineStr">
+        <is>
+          <t>yc</t>
+        </is>
+      </c>
+      <c r="I5" s="41" t="n">
         <v>6</v>
       </c>
-      <c r="J5" s="29" t="n">
+      <c r="J5" s="41" t="n">
         <v>6</v>
       </c>
-      <c r="K5" s="29" t="n">
+      <c r="K5" s="41" t="n">
         <v>4</v>
       </c>
-      <c r="L5" s="33" t="n"/>
-      <c r="M5" s="33" t="n"/>
+      <c r="L5" s="46" t="n"/>
+      <c r="M5" s="46" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="12" t="n">

</xml_diff>